<commit_message>
Status tracker after batch 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E143B9FF-F8F5-477A-BDC9-00C4484CD24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0197CF2A-425D-4026-8ABF-B2047D22162A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="351">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -154,7 +154,7 @@
     <t>2026-10-02</t>
   </si>
   <si>
-    <t>Built. Only 5 units, all process-scale (Carr Centritech Centritec Cell 8, Sharples Type 1P, a beaker centrifuge), not benchtop instruments; the copy says so. 'lab centrifuge' and 'ultracentrifuge' demand is lab-instrument (Beckman, Thermo), so the ultracentrifuge terms are excluded. No size or condition tabs (all used).</t>
+    <t>Built. Only 5 units, all process-scale (Carr Centritech Centritec Cell 8, Sharples Type 1P, a beaker centrifuge), not benchtop instruments; the copy says so. 'lab centrifuge' and 'ultracentrifuge' demand is lab-instrument (Beckman, Thermo), so the ultracentrifuge terms are excluded. No size or condition tabs (all used). 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
   </si>
   <si>
     <t>2</t>
@@ -181,7 +181,7 @@
     <t>equipment/centrifuge/misc-and-hydraulic-centrifuge/INTERNAL-REVIEW-misc-and-hydraulic-centrifuge.html</t>
   </si>
   <si>
-    <t>Built as 'Tubular, Podbielniak &amp; Hydraulic Centrifuges': IMS's misc bucket is Sharples tubular super centrifuges, Podbielniak extractors and hydraulic drives. 'Hydraulic centrifuge' has no search demand; the page targets tubular / super / sharples / centrifugal extractor.</t>
+    <t>Built as 'Tubular, Podbielniak &amp; Hydraulic Centrifuges': IMS's misc bucket is Sharples tubular super centrifuges, Podbielniak extractors and hydraulic drives. 'Hydraulic centrifuge' has no search demand; the page targets tubular / super / sharples / centrifugal extractor. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
   </si>
   <si>
     <t>3</t>
@@ -208,7 +208,7 @@
     <t>equipment/centrifuge/peeler-centrifuge/INTERNAL-REVIEW-peeler-centrifuge.html</t>
   </si>
   <si>
-    <t>Built. IPP's blog already ranks for 'what is a peeler centrifuge' and 'peeler vs pusher', so the FAQ answers briefly and links to those guides.</t>
+    <t>Built. IPP's blog already ranks for 'what is a peeler centrifuge' and 'peeler vs pusher', so the FAQ answers briefly and links to those guides. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
   </si>
   <si>
     <t>4</t>
@@ -238,7 +238,7 @@
     <t>equipment/centrifuge/pusher-centrifuge-parts/INTERNAL-REVIEW-pusher-centrifuge-parts.html</t>
   </si>
   <si>
-    <t>Built. 21 parts listings, only 1 with a photo, mostly Krauss Maffei SB1000/2 components. Part type comes from the IMS description, and browse cards use IMS keyword search. Generic 'centrifuge parts' demand is lab-instrument parts, so it is excluded.</t>
+    <t>Built. 21 parts listings, only 1 with a photo, mostly Krauss Maffei SB1000/2 components. Part type comes from the IMS description, and browse cards use IMS keyword search. Generic 'centrifuge parts' demand is lab-instrument parts, so it is excluded. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
   </si>
   <si>
     <t>5</t>
@@ -262,7 +262,7 @@
     <t>equipment/centrifuge/pusher-centrifuge/INTERNAL-REVIEW-pusher-centrifuge.html</t>
   </si>
   <si>
-    <t>Built from 26 complete machines (the 21 parts-only listings are on priority 4). The IMS 'Browse All' links show IMS's own pusher search, which includes the parts.</t>
+    <t>Built from 26 complete machines (the 21 parts-only listings are on priority 4). The IMS 'Browse All' links show IMS's own pusher search, which includes the parts. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
   </si>
   <si>
     <t>6</t>
@@ -280,114 +280,153 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/solid-bowl-decanter-centrifuge/parts-only</t>
   </si>
   <si>
+    <t>decanter centrifuge parts</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/centrifuge/solid-bowl-decanter-centrifuge-parts/</t>
+  </si>
+  <si>
+    <t>equipment/centrifuge/solid-bowl-decanter-centrifuge-parts/INTERNAL-REVIEW-solid-bowl-decanter-centrifuge-parts.html</t>
+  </si>
+  <si>
+    <t>Built. 7 parts listings, all with photos: scroll conveyors (Sharples P3400, Alfa Laval NX314, Dorr Oliver for the 16L and Z3L), Sharples P-2000 and Sangerhausen rotating assemblies, and a Bird gearbox. Part type comes from the IMS description. Complete-machine and repair queries are excluded (the live decanter page owns machines).</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Dryer- Nauta / Conical</t>
+  </si>
+  <si>
+    <t>Nauta Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/nauta-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/nauta-dryer</t>
+  </si>
+  <si>
+    <t>nauta dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/nauta-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/nauta-dryer/INTERNAL-REVIEW-nauta-dryer.html</t>
+  </si>
+  <si>
+    <t>Built. 11 units from 9 OEMs (Krauss Maffei, Bolz, Vrieco Nauta, Hosokawa Alpine and others). Nauta mixer terms are excluded (the live Nauta mixer page owns them); double cone terms belong to the twin shell page, linked from the comparison table.</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Dryer-Drum</t>
+  </si>
+  <si>
+    <t>Drum Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/drum-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/drum-dryer</t>
+  </si>
+  <si>
+    <t>drum dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/drum-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/drum-dryer/INTERNAL-REVIEW-drum-dryer.html</t>
+  </si>
+  <si>
+    <t>Built. 16 listings: Simon Dryers, Blaw Knox and Gouda single and double drum dryers plus unused spare drums. Household laundry dryer and rotary drum dryer terms are excluded.</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Dryer-Flash</t>
+  </si>
+  <si>
+    <t>Flash Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/flash-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/flash-dryer</t>
+  </si>
+  <si>
+    <t>industrial flash dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/flash-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/flash-dryer/INTERNAL-REVIEW-flash-dryer.html</t>
+  </si>
+  <si>
+    <t>Built (new URL, no live page). Only 4 units: APV Anhydro spin flash, Aljet, Hosokawa Alpine MDV-4, AKSH Engineering. Screen-printing flash dryers dominate 'flash dryer' demand, so the H1 says industrial. The IMS inlet-moisture fields and the Hosokawa evaporation field are mislabelled, so they are not published.</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Dryer-Porcupine</t>
+  </si>
+  <si>
+    <t>Parts</t>
+  </si>
+  <si>
+    <t>Porcupine Dryer Parts</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/porcupine-dryer-parts/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/porcupine-dryer/parts</t>
+  </si>
+  <si>
+    <t>porcupine dryer parts</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/porcupine-dryer-parts/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/porcupine-dryer-parts/INTERNAL-REVIEW-porcupine-dryer-parts.html</t>
+  </si>
+  <si>
+    <t>Built (new URL). 4 GPS listings: 3 troughs and a new shaft and flights set. 'porcupine dryer' demand belongs to the live porcupine dryer page, linked from an FAQ. Parts queries have no measured volume. The GPS/Bethlehem brand angle comes from IPP's own news post (not linked).</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Dryer-Rotary Hot Air</t>
+  </si>
+  <si>
+    <t>Rotary Hot Air Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/rotary-hot-air-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/rotary-hot-air-dryer</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>equipment/centrifuge/solid-bowl-decanter-centrifuge-parts/INTERNAL-REVIEW-solid-bowl-decanter-centrifuge-parts.html</t>
-  </si>
-  <si>
-    <t>7 parts listings on IMS.</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>Dryer- Nauta / Conical</t>
-  </si>
-  <si>
-    <t>Nauta Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/nauta-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/nauta-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/nauta-dryer/INTERNAL-REVIEW-nauta-dryer.html</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>Dryer-Drum</t>
-  </si>
-  <si>
-    <t>Drum Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/drum-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/drum-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/drum-dryer/INTERNAL-REVIEW-drum-dryer.html</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>Dryer-Flash</t>
-  </si>
-  <si>
-    <t>Flash Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/flash-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/flash-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/flash-dryer/INTERNAL-REVIEW-flash-dryer.html</t>
+    <t>equipment/dryer/rotary-hot-air-dryer/INTERNAL-REVIEW-rotary-hot-air-dryer.html</t>
   </si>
   <si>
     <t>Thin inventory: 4 units.</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Dryer-Porcupine</t>
-  </si>
-  <si>
-    <t>Parts</t>
-  </si>
-  <si>
-    <t>Porcupine Dryer Parts</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/porcupine-dryer-parts/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/porcupine-dryer/parts</t>
-  </si>
-  <si>
-    <t>equipment/dryer/porcupine-dryer-parts/INTERNAL-REVIEW-porcupine-dryer-parts.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 4 listings.</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>Dryer-Rotary Hot Air</t>
-  </si>
-  <si>
-    <t>Rotary Hot Air Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/rotary-hot-air-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/rotary-hot-air-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/rotary-hot-air-dryer/INTERNAL-REVIEW-rotary-hot-air-dryer.html</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
@@ -625,10 +664,7 @@
     <t>equipment/heat-exchanger/plate-and-frame/INTERNAL-REVIEW-plate-and-frame.html</t>
   </si>
   <si>
-    <t>2026-10-01</t>
-  </si>
-  <si>
-    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages.</t>
+    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
   </si>
   <si>
     <t>23</t>
@@ -1681,7 +1717,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -1757,7 +1793,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>39</v>
       </c>
@@ -1833,7 +1869,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="51" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>48</v>
       </c>
@@ -1909,7 +1945,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>57</v>
       </c>
@@ -1987,7 +2023,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>67</v>
       </c>
@@ -2063,7 +2099,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>75</v>
       </c>
@@ -2088,320 +2124,382 @@
       <c r="H10" s="3">
         <v>7</v>
       </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="3"/>
+      <c r="I10" s="3">
+        <v>7</v>
+      </c>
+      <c r="J10" s="3">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="L10" s="3">
+        <v>10</v>
+      </c>
       <c r="M10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="T10" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U10" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V10" s="4"/>
+      <c r="V10" s="5" t="s">
+        <v>81</v>
+      </c>
       <c r="W10" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="X10" s="4"/>
+        <v>82</v>
+      </c>
+      <c r="X10" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y10" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B11" s="3">
         <v>2</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H11" s="3">
         <v>11</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="3"/>
+      <c r="I11" s="3">
+        <v>11</v>
+      </c>
+      <c r="J11" s="3">
+        <v>11</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="L11" s="3">
+        <v>150</v>
+      </c>
       <c r="M11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="R11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="T11" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U11" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V11" s="4"/>
+      <c r="V11" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="W11" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="7"/>
-    </row>
-    <row r="12" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="X11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y11" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B12" s="3">
         <v>2</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H12" s="3">
         <v>16</v>
       </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="3"/>
+      <c r="I12" s="3">
+        <v>16</v>
+      </c>
+      <c r="J12" s="3">
+        <v>16</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L12" s="3">
+        <v>300</v>
+      </c>
       <c r="M12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="R12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="T12" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U12" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V12" s="4"/>
+      <c r="V12" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="W12" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="X12" s="4"/>
-      <c r="Y12" s="7"/>
-    </row>
-    <row r="13" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y12" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B13" s="3">
         <v>2</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="H13" s="3">
         <v>4</v>
       </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="3"/>
+      <c r="I13" s="3">
+        <v>4</v>
+      </c>
+      <c r="J13" s="3">
+        <v>4</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="L13" s="3">
+        <v>40</v>
+      </c>
       <c r="M13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="R13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="T13" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V13" s="4"/>
+      <c r="V13" s="5" t="s">
+        <v>108</v>
+      </c>
       <c r="W13" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="X13" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y13" s="7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="B14" s="3">
         <v>2</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H14" s="3">
         <v>4</v>
       </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="4"/>
+      <c r="I14" s="3">
+        <v>4</v>
+      </c>
+      <c r="J14" s="3">
+        <v>2</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>117</v>
+      </c>
       <c r="L14" s="3"/>
       <c r="M14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="R14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="T14" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U14" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V14" s="4"/>
+      <c r="V14" s="5" t="s">
+        <v>118</v>
+      </c>
       <c r="W14" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="X14" s="4"/>
+        <v>119</v>
+      </c>
+      <c r="X14" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y14" s="7" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="B15" s="3">
         <v>3</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="H15" s="3">
         <v>4</v>
@@ -2411,25 +2509,25 @@
       <c r="K15" s="4"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T15" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2440,32 +2538,32 @@
       </c>
       <c r="V15" s="4"/>
       <c r="W15" s="4" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="X15" s="4"/>
       <c r="Y15" s="7" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="B16" s="3">
         <v>3</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="H16" s="3">
         <v>32</v>
@@ -2475,25 +2573,25 @@
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T16" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2504,32 +2602,32 @@
       </c>
       <c r="V16" s="4"/>
       <c r="W16" s="4" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="X16" s="4"/>
       <c r="Y16" s="7" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="B17" s="3">
         <v>3</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="H17" s="3">
         <v>15</v>
@@ -2539,25 +2637,25 @@
       <c r="K17" s="4"/>
       <c r="L17" s="3"/>
       <c r="M17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T17" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2568,30 +2666,30 @@
       </c>
       <c r="V17" s="4"/>
       <c r="W17" s="4" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="X17" s="4"/>
       <c r="Y17" s="7"/>
     </row>
     <row r="18" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="H18" s="3">
         <v>8</v>
@@ -2601,25 +2699,25 @@
       <c r="K18" s="4"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T18" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2630,30 +2728,30 @@
       </c>
       <c r="V18" s="4"/>
       <c r="W18" s="4" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="X18" s="4"/>
       <c r="Y18" s="7"/>
     </row>
     <row r="19" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="B19" s="3">
         <v>3</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="H19" s="3">
         <v>3</v>
@@ -2663,25 +2761,25 @@
       <c r="K19" s="4"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T19" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2692,32 +2790,32 @@
       </c>
       <c r="V19" s="4"/>
       <c r="W19" s="4" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="X19" s="4"/>
       <c r="Y19" s="7" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="B20" s="3">
         <v>4</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="H20" s="3">
         <v>7</v>
@@ -2727,25 +2825,25 @@
       <c r="K20" s="4"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2756,30 +2854,30 @@
       </c>
       <c r="V20" s="4"/>
       <c r="W20" s="4" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="X20" s="4"/>
       <c r="Y20" s="7"/>
     </row>
     <row r="21" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="B21" s="3">
         <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="H21" s="3">
         <v>11</v>
@@ -2789,25 +2887,25 @@
       <c r="K21" s="4"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T21" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2818,30 +2916,30 @@
       </c>
       <c r="V21" s="4"/>
       <c r="W21" s="4" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="X21" s="4"/>
       <c r="Y21" s="7"/>
     </row>
     <row r="22" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="B22" s="3">
         <v>4</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="H22" s="3">
         <v>24</v>
@@ -2851,25 +2949,25 @@
       <c r="K22" s="4"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T22" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2880,32 +2978,32 @@
       </c>
       <c r="V22" s="4"/>
       <c r="W22" s="4" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="7"/>
     </row>
     <row r="23" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="B23" s="3">
         <v>4</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="H23" s="3">
         <v>4</v>
@@ -2915,25 +3013,25 @@
       <c r="K23" s="4"/>
       <c r="L23" s="3"/>
       <c r="M23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T23" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2944,34 +3042,34 @@
       </c>
       <c r="V23" s="4"/>
       <c r="W23" s="4" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="7" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B24" s="3">
         <v>4</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="H24" s="3">
         <v>12</v>
@@ -2981,25 +3079,25 @@
       <c r="K24" s="4"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T24" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3010,32 +3108,32 @@
       </c>
       <c r="V24" s="4"/>
       <c r="W24" s="4" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="7"/>
     </row>
     <row r="25" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="B25" s="3">
         <v>5</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="H25" s="3">
         <v>5</v>
@@ -3045,25 +3143,25 @@
       <c r="K25" s="4"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3074,34 +3172,34 @@
       </c>
       <c r="V25" s="4"/>
       <c r="W25" s="4" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="7" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="26" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B26" s="3">
         <v>5</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="H26" s="3">
         <v>94</v>
@@ -3111,25 +3209,25 @@
       <c r="K26" s="4"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3140,32 +3238,32 @@
       </c>
       <c r="V26" s="4"/>
       <c r="W26" s="4" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="X26" s="4"/>
       <c r="Y26" s="7"/>
     </row>
-    <row r="27" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="51" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="B27" s="3">
         <v>0</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="H27" s="3">
         <v>161</v>
@@ -3177,7 +3275,7 @@
         <v>148</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="L27" s="3">
         <v>1100</v>
@@ -3211,39 +3309,39 @@
         <v>34</v>
       </c>
       <c r="V27" s="5" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="W27" s="4" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="X27" s="4" t="s">
-        <v>195</v>
+        <v>37</v>
       </c>
       <c r="Y27" s="7" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="B28" s="3">
         <v>5</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="H28" s="3">
         <v>67</v>
@@ -3253,25 +3351,25 @@
       <c r="K28" s="4"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3282,32 +3380,32 @@
       </c>
       <c r="V28" s="4"/>
       <c r="W28" s="4" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="X28" s="4"/>
       <c r="Y28" s="7"/>
     </row>
     <row r="29" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B29" s="3">
         <v>5</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="H29" s="3">
         <v>31</v>
@@ -3317,25 +3415,25 @@
       <c r="K29" s="4"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T29" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3346,30 +3444,30 @@
       </c>
       <c r="V29" s="4"/>
       <c r="W29" s="4" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="X29" s="4"/>
       <c r="Y29" s="7"/>
     </row>
     <row r="30" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="B30" s="3">
         <v>5</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="H30" s="3">
         <v>5</v>
@@ -3379,25 +3477,25 @@
       <c r="K30" s="4"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T30" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3408,32 +3506,32 @@
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="4" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="7" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="31" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B31" s="3">
         <v>6</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="H31" s="3">
         <v>1</v>
@@ -3443,25 +3541,25 @@
       <c r="K31" s="4"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T31" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3472,32 +3570,32 @@
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="4" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="7" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
     </row>
     <row r="32" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="H32" s="3">
         <v>2</v>
@@ -3507,25 +3605,25 @@
       <c r="K32" s="4"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T32" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3536,32 +3634,32 @@
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="4" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="7" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="33" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="B33" s="3">
         <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="H33" s="3">
         <v>2</v>
@@ -3571,25 +3669,25 @@
       <c r="K33" s="4"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3600,34 +3698,34 @@
       </c>
       <c r="V33" s="4"/>
       <c r="W33" s="4" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="X33" s="4"/>
       <c r="Y33" s="7" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="34" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="B34" s="3">
         <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="H34" s="3">
         <v>8</v>
@@ -3637,25 +3735,25 @@
       <c r="K34" s="4"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3666,32 +3764,32 @@
       </c>
       <c r="V34" s="4"/>
       <c r="W34" s="4" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="X34" s="4"/>
       <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="B35" s="3">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="H35" s="3">
         <v>14</v>
@@ -3701,25 +3799,25 @@
       <c r="K35" s="4"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T35" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3730,32 +3828,32 @@
       </c>
       <c r="V35" s="4"/>
       <c r="W35" s="4" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="X35" s="4"/>
       <c r="Y35" s="7"/>
     </row>
     <row r="36" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B36" s="3">
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="H36" s="3">
         <v>1</v>
@@ -3765,25 +3863,25 @@
       <c r="K36" s="4"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3794,34 +3892,34 @@
       </c>
       <c r="V36" s="4"/>
       <c r="W36" s="4" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="X36" s="4"/>
       <c r="Y36" s="7" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B37" s="3">
         <v>7</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
@@ -3831,25 +3929,25 @@
       <c r="K37" s="4"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3860,34 +3958,34 @@
       </c>
       <c r="V37" s="4"/>
       <c r="W37" s="4" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="X37" s="4"/>
       <c r="Y37" s="7" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="B38" s="3">
         <v>7</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="H38" s="3">
         <v>2</v>
@@ -3897,25 +3995,25 @@
       <c r="K38" s="4"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3926,34 +4024,34 @@
       </c>
       <c r="V38" s="4"/>
       <c r="W38" s="4" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="X38" s="4"/>
       <c r="Y38" s="7" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="B39" s="3">
         <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="H39" s="3">
         <v>6</v>
@@ -3963,25 +4061,25 @@
       <c r="K39" s="4"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3992,32 +4090,32 @@
       </c>
       <c r="V39" s="4"/>
       <c r="W39" s="4" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="X39" s="4"/>
       <c r="Y39" s="7"/>
     </row>
     <row r="40" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="B40" s="3">
         <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="H40" s="3">
         <v>33</v>
@@ -4027,25 +4125,25 @@
       <c r="K40" s="4"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T40" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4056,32 +4154,32 @@
       </c>
       <c r="V40" s="4"/>
       <c r="W40" s="4" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="X40" s="4"/>
       <c r="Y40" s="7" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
     </row>
     <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="B41" s="3">
         <v>8</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="H41" s="3">
         <v>9</v>
@@ -4091,25 +4189,25 @@
       <c r="K41" s="4"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4120,30 +4218,30 @@
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="X41" s="4"/>
       <c r="Y41" s="7"/>
     </row>
     <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
@@ -4153,25 +4251,25 @@
       <c r="K42" s="4"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4182,32 +4280,32 @@
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="X42" s="4"/>
       <c r="Y42" s="7" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
@@ -4217,25 +4315,25 @@
       <c r="K43" s="4"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4246,32 +4344,32 @@
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="X43" s="4"/>
       <c r="Y43" s="7" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
@@ -4281,25 +4379,25 @@
       <c r="K44" s="4"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4310,11 +4408,11 @@
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="X44" s="4"/>
       <c r="Y44" s="7" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -4379,75 +4477,80 @@
     <hyperlink ref="V9" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="F10" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
     <hyperlink ref="G10" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="F11" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="G11" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="F12" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="G12" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="F13" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="G13" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="F14" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="G14" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="F15" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="G15" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="F16" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="G16" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="F17" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="G17" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="F18" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="G18" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="F19" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="G19" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="F20" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="G20" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="F21" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="G21" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="F22" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="G22" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="F23" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="G23" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="F24" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="G24" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="F25" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="G25" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="F26" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="G26" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="F27" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="G27" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="V27" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="F28" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="G28" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="F29" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="G29" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="F30" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="G30" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="F31" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="G31" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="F32" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="G32" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="F33" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="G33" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="F34" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="G34" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="F35" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="G35" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="F36" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="G36" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="F37" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="G37" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="F38" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="G38" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="F39" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="G39" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="F40" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="G40" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="F41" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="G41" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="F42" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="G42" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="F43" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="G43" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="F44" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="G44" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="V10" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="F11" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="G11" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="V11" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="F12" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="G12" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="V12" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="F13" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="G13" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="V13" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="F14" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="G14" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="V14" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="F15" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="G15" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="F16" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="G16" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="F17" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="G17" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="F18" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="G18" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="F19" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="G19" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="F20" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="G20" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="F21" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="G21" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="F22" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="G22" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="F23" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="G23" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="F24" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="G24" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="F25" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="G25" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="F26" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="G26" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="F27" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="G27" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="V27" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="F28" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="G28" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="F29" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="G29" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="F30" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="G30" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="F31" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="G31" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="F32" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="G32" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="F33" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="G33" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="F34" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="G34" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="F35" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="G35" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="F36" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="G36" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="F37" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="G37" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="F38" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="G38" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="F39" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="G39" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="F40" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="G40" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="F41" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="G41" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="F42" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="G42" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="F43" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="G43" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="F44" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="G44" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4467,25 +4570,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -4494,16 +4597,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -4512,16 +4615,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -4530,7 +4633,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -4539,7 +4642,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -4548,27 +4651,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>300</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4577,11 +4680,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -4590,11 +4693,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -4603,11 +4706,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4616,11 +4719,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -4629,11 +4732,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -4642,11 +4745,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -4655,16 +4758,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.27500000000000002</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -4672,16 +4775,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -4736,7 +4839,7 @@
       </c>
       <c r="C28" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A28,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D28" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A28,Pages!$U$5:$U$44,"Approved")</f>
@@ -4744,7 +4847,7 @@
       </c>
       <c r="E28" s="6" t="str">
         <f>IF(D28=B28,"Approved",IF(C28=B28,"Ready for client review",IF(C28&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A28,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -4889,15 +4992,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -4905,7 +5008,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4913,7 +5016,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -4921,7 +5024,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -4929,7 +5032,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4937,7 +5040,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -4945,7 +5048,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -4953,7 +5056,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -4961,28 +5064,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Tracker: batch 3 (P11-15) ready for client review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0197CF2A-425D-4026-8ABF-B2047D22162A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67B4A47-6B94-4D9D-A200-2DC5B1B85C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="364">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -154,7 +154,7 @@
     <t>2026-10-02</t>
   </si>
   <si>
-    <t>Built. Only 5 units, all process-scale (Carr Centritech Centritec Cell 8, Sharples Type 1P, a beaker centrifuge), not benchtop instruments; the copy says so. 'lab centrifuge' and 'ultracentrifuge' demand is lab-instrument (Beckman, Thermo), so the ultracentrifuge terms are excluded. No size or condition tabs (all used). 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
+    <t>Built. Only 5 units, all process-scale (Carr Centritech Centritec Cell 8, Sharples Type 1P, a beaker centrifuge), not benchtop instruments; the copy says so. 'lab centrifuge' and 'ultracentrifuge' demand is lab-instrument (Beckman, Thermo), so the ultracentrifuge terms are excluded. No size or condition tabs (all used). 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>2</t>
@@ -181,7 +181,7 @@
     <t>equipment/centrifuge/misc-and-hydraulic-centrifuge/INTERNAL-REVIEW-misc-and-hydraulic-centrifuge.html</t>
   </si>
   <si>
-    <t>Built as 'Tubular, Podbielniak &amp; Hydraulic Centrifuges': IMS's misc bucket is Sharples tubular super centrifuges, Podbielniak extractors and hydraulic drives. 'Hydraulic centrifuge' has no search demand; the page targets tubular / super / sharples / centrifugal extractor. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
+    <t>Built as 'Tubular, Podbielniak &amp; Hydraulic Centrifuges': IMS's misc bucket is Sharples tubular super centrifuges, Podbielniak extractors and hydraulic drives. 'Hydraulic centrifuge' has no search demand; the page targets tubular / super / sharples / centrifugal extractor. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>3</t>
@@ -208,7 +208,7 @@
     <t>equipment/centrifuge/peeler-centrifuge/INTERNAL-REVIEW-peeler-centrifuge.html</t>
   </si>
   <si>
-    <t>Built. IPP's blog already ranks for 'what is a peeler centrifuge' and 'peeler vs pusher', so the FAQ answers briefly and links to those guides. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
+    <t>Built. IPP's blog already ranks for 'what is a peeler centrifuge' and 'peeler vs pusher', so the FAQ answers briefly and links to those guides. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>4</t>
@@ -238,7 +238,7 @@
     <t>equipment/centrifuge/pusher-centrifuge-parts/INTERNAL-REVIEW-pusher-centrifuge-parts.html</t>
   </si>
   <si>
-    <t>Built. 21 parts listings, only 1 with a photo, mostly Krauss Maffei SB1000/2 components. Part type comes from the IMS description, and browse cards use IMS keyword search. Generic 'centrifuge parts' demand is lab-instrument parts, so it is excluded. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
+    <t>Built. 21 parts listings, only 1 with a photo, mostly Krauss Maffei SB1000/2 components. Part type comes from the IMS description, and browse cards use IMS keyword search. Generic 'centrifuge parts' demand is lab-instrument parts, so it is excluded. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>5</t>
@@ -262,7 +262,7 @@
     <t>equipment/centrifuge/pusher-centrifuge/INTERNAL-REVIEW-pusher-centrifuge.html</t>
   </si>
   <si>
-    <t>Built from 26 complete machines (the 21 parts-only listings are on priority 4). The IMS 'Browse All' links show IMS's own pusher search, which includes the parts. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
+    <t>Built from 26 complete machines (the 21 parts-only listings are on priority 4). The IMS 'Browse All' links show IMS's own pusher search, which includes the parts. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>6</t>
@@ -289,7 +289,7 @@
     <t>equipment/centrifuge/solid-bowl-decanter-centrifuge-parts/INTERNAL-REVIEW-solid-bowl-decanter-centrifuge-parts.html</t>
   </si>
   <si>
-    <t>Built. 7 parts listings, all with photos: scroll conveyors (Sharples P3400, Alfa Laval NX314, Dorr Oliver for the 16L and Z3L), Sharples P-2000 and Sangerhausen rotating assemblies, and a Bird gearbox. Part type comes from the IMS description. Complete-machine and repair queries are excluded (the live decanter page owns machines).</t>
+    <t>Built. 7 parts listings, all with photos: scroll conveyors (Sharples P3400, Alfa Laval NX314, Dorr Oliver for the 16L and Z3L), Sharples P-2000 and Sangerhausen rotating assemblies, and a Bird gearbox. Part type comes from the IMS description. Complete-machine and repair queries are excluded (the live decanter page owns machines). Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>7</t>
@@ -316,7 +316,7 @@
     <t>equipment/dryer/nauta-dryer/INTERNAL-REVIEW-nauta-dryer.html</t>
   </si>
   <si>
-    <t>Built. 11 units from 9 OEMs (Krauss Maffei, Bolz, Vrieco Nauta, Hosokawa Alpine and others). Nauta mixer terms are excluded (the live Nauta mixer page owns them); double cone terms belong to the twin shell page, linked from the comparison table.</t>
+    <t>Built. 11 units from 9 OEMs (Krauss Maffei, Bolz, Vrieco Nauta, Hosokawa Alpine and others). Nauta mixer terms are excluded (the live Nauta mixer page owns them); double cone terms belong to the twin shell page, linked from the comparison table. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>8</t>
@@ -343,7 +343,7 @@
     <t>equipment/dryer/drum-dryer/INTERNAL-REVIEW-drum-dryer.html</t>
   </si>
   <si>
-    <t>Built. 16 listings: Simon Dryers, Blaw Knox and Gouda single and double drum dryers plus unused spare drums. Household laundry dryer and rotary drum dryer terms are excluded.</t>
+    <t>Built. 16 listings: Simon Dryers, Blaw Knox and Gouda single and double drum dryers plus unused spare drums. Household laundry dryer and rotary drum dryer terms are excluded. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>9</t>
@@ -370,7 +370,7 @@
     <t>equipment/dryer/flash-dryer/INTERNAL-REVIEW-flash-dryer.html</t>
   </si>
   <si>
-    <t>Built (new URL, no live page). Only 4 units: APV Anhydro spin flash, Aljet, Hosokawa Alpine MDV-4, AKSH Engineering. Screen-printing flash dryers dominate 'flash dryer' demand, so the H1 says industrial. The IMS inlet-moisture fields and the Hosokawa evaporation field are mislabelled, so they are not published.</t>
+    <t>Built (new URL, no live page). Only 4 units: APV Anhydro spin flash, Aljet, Hosokawa Alpine MDV-4, AKSH Engineering. Screen-printing flash dryers dominate 'flash dryer' demand, so the H1 says industrial. The IMS inlet-moisture fields and the Hosokawa evaporation field are mislabelled, so they are not published. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>10</t>
@@ -400,7 +400,7 @@
     <t>equipment/dryer/porcupine-dryer-parts/INTERNAL-REVIEW-porcupine-dryer-parts.html</t>
   </si>
   <si>
-    <t>Built (new URL). 4 GPS listings: 3 troughs and a new shaft and flights set. 'porcupine dryer' demand belongs to the live porcupine dryer page, linked from an FAQ. Parts queries have no measured volume. The GPS/Bethlehem brand angle comes from IPP's own news post (not linked).</t>
+    <t>Built (new URL). 4 GPS listings: 3 troughs and a new shaft and flights set. 'porcupine dryer' demand belongs to the live porcupine dryer page, linked from an FAQ. Parts queries have no measured volume. The GPS/Bethlehem brand angle comes from IPP's own news post (not linked). Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>11</t>
@@ -418,168 +418,207 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/rotary-hot-air-dryer</t>
   </si>
   <si>
+    <t>rotary dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/rotary-hot-air-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/rotary-hot-air-dryer/INTERNAL-REVIEW-rotary-hot-air-dryer.html</t>
+  </si>
+  <si>
+    <t>Built from 4 units: a Standard Steel louver dryer and a Patterson Kelly unit in stainless steel 304, a Link Belt in carbon steel, and a refurbished stainless steel 316 co-current dryer. The refurbished listing says both 'direct fired' and steam; the copy uses steam. Comparison links to the live rotary steam tube dryer page. Manufacturer, design, maintenance, triple-pass and household vent terms excluded.</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Dryer-Shelf</t>
+  </si>
+  <si>
+    <t>Shelf Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/shelf-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/shelf-dryer</t>
+  </si>
+  <si>
+    <t>vacuum tray dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/shelf-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/shelf-dryer/INTERNAL-REVIEW-shelf-dryer.html</t>
+  </si>
+  <si>
+    <t>Built from 23 listings: 22 good used vacuum shelf and tray dryers and a new GPS vacuum tray dryer. The IMS shelf-dryer search also returns oven dryers; they stay off the page. The Stokes hot water generator is described as an accessory. Unit defect notes and mis-entered IMS dimensions are not repeated. The IMS Leybold manufacturer filter is broken (returns all 32), so Leybold has no tab. Pharmaceutical, rotary tray, household and parts terms excluded.</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Dryer-Thin Film</t>
+  </si>
+  <si>
+    <t>Thin Film Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/thin-film-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/thin-film-dryer</t>
+  </si>
+  <si>
+    <t>thin film dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/thin-film-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/thin-film-dryer/INTERNAL-REVIEW-thin-film-dryer.html</t>
+  </si>
+  <si>
+    <t>Built from 15 units: Luwa SMS DK600, D-850 and 1000/6000 dryers and a Buss-SMS-Canzler D-015, all stainless. IMS lists the DK600 units as coolers; an FAQ covers cooling duty. Thin film evaporator terms are excluded (IPP's evaporator page and blog own them); the comparison links to the live evaporator page.</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Dryer-Thermal Disc</t>
+  </si>
+  <si>
+    <t>Thermal Disc Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/thermal-disc-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/thermal-disc-dryer</t>
+  </si>
+  <si>
+    <t>horizontal disc dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/thermal-disc-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/thermal-disc-dryer/INTERNAL-REVIEW-thermal-disc-dryer.html</t>
+  </si>
+  <si>
+    <t>Built from 8 units: unused surplus Bepex TorusDisc TD48-9 units, a Bepex Model 60-14, a Bethlehem processor and a Strong Scott TDJ. IMS lists the TD48-9 units as coolers; unit 239472 has no IMS data. Comparison links to the live porcupine dryer page. Sludge, rendering and fish meal (application) terms excluded.</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Dryer-Spherical</t>
+  </si>
+  <si>
+    <t>Spherical Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/spherical-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/spherical-dryer</t>
+  </si>
+  <si>
+    <t>spherical dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/spherical-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/spherical-dryer/INTERNAL-REVIEW-spherical-dryer.html</t>
+  </si>
+  <si>
+    <t>Built from 3 units: two Rosenmund AG RKT-2000 dryers and a Pierre Guerin Turbosphere TS200, jacketed, stainless steel 316L. Rosenmund vessel and jacket pressures are not published (the IMS fields look swapped or inconsistent) and the IMS model field holds the town. The comparison links to the Nauta dryer page, which is new and not live yet, so publish them together.</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>Dryer-Pan</t>
+  </si>
+  <si>
+    <t>Pan Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/pan-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/pan-dryer</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>equipment/dryer/rotary-hot-air-dryer/INTERNAL-REVIEW-rotary-hot-air-dryer.html</t>
+    <t>equipment/dryer/pan-dryer/INTERNAL-REVIEW-pan-dryer.html</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Dryer-Oven</t>
+  </si>
+  <si>
+    <t>Oven Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/oven-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/oven-dryer</t>
+  </si>
+  <si>
+    <t>equipment/dryer/oven-dryer/INTERNAL-REVIEW-oven-dryer.html</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>Dryer-Flaker Drum and Belt</t>
+  </si>
+  <si>
+    <t>Flaker Drum and Belt Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/flaker-drum-and-belt-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/flaker-drum-and-belt-dryer</t>
+  </si>
+  <si>
+    <t>equipment/dryer/flaker-drum-and-belt-dryer/INTERNAL-REVIEW-flaker-drum-and-belt-dryer.html</t>
+  </si>
+  <si>
+    <t>19a</t>
+  </si>
+  <si>
+    <t>Dryer-Air</t>
+  </si>
+  <si>
+    <t>Desiccant</t>
+  </si>
+  <si>
+    <t>Desiccant Air Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/desiccant/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/air-dryer/desiccant</t>
+  </si>
+  <si>
+    <t>equipment/dryer/desiccant/INTERNAL-REVIEW-desiccant.html</t>
   </si>
   <si>
     <t>Thin inventory: 4 units.</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>Dryer-Shelf</t>
-  </si>
-  <si>
-    <t>Shelf Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/shelf-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/shelf-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/shelf-dryer/INTERNAL-REVIEW-shelf-dryer.html</t>
-  </si>
-  <si>
-    <t>The IMS shelf-dryer search also returns oven dryers (32 listings in total); only true shelf dryers will appear on the page.</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>Dryer-Thin Film</t>
-  </si>
-  <si>
-    <t>Thin Film Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/thin-film-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/thin-film-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/thin-film-dryer/INTERNAL-REVIEW-thin-film-dryer.html</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Dryer-Thermal Disc</t>
-  </si>
-  <si>
-    <t>Thermal Disc Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/thermal-disc-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/thermal-disc-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/thermal-disc-dryer/INTERNAL-REVIEW-thermal-disc-dryer.html</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Dryer-Spherical</t>
-  </si>
-  <si>
-    <t>Spherical Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/spherical-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/spherical-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/spherical-dryer/INTERNAL-REVIEW-spherical-dryer.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 3 units.</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>Dryer-Pan</t>
-  </si>
-  <si>
-    <t>Pan Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/pan-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/pan-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/pan-dryer/INTERNAL-REVIEW-pan-dryer.html</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>Dryer-Oven</t>
-  </si>
-  <si>
-    <t>Oven Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/oven-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/oven-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/oven-dryer/INTERNAL-REVIEW-oven-dryer.html</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>Dryer-Flaker Drum and Belt</t>
-  </si>
-  <si>
-    <t>Flaker Drum and Belt Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/flaker-drum-and-belt-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/flaker-drum-and-belt-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/flaker-drum-and-belt-dryer/INTERNAL-REVIEW-flaker-drum-and-belt-dryer.html</t>
-  </si>
-  <si>
-    <t>19a</t>
-  </si>
-  <si>
-    <t>Dryer-Air</t>
-  </si>
-  <si>
-    <t>Desiccant</t>
-  </si>
-  <si>
-    <t>Desiccant Air Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/desiccant/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/air-dryer/desiccant</t>
-  </si>
-  <si>
-    <t>equipment/dryer/desiccant/INTERNAL-REVIEW-desiccant.html</t>
-  </si>
-  <si>
     <t>19b</t>
   </si>
   <si>
@@ -664,7 +703,7 @@
     <t>equipment/heat-exchanger/plate-and-frame/INTERNAL-REVIEW-plate-and-frame.html</t>
   </si>
   <si>
-    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied.</t>
+    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
   </si>
   <si>
     <t>23</t>
@@ -1717,7 +1756,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -1793,7 +1832,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>39</v>
       </c>
@@ -1869,7 +1908,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>48</v>
       </c>
@@ -1945,7 +1984,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>57</v>
       </c>
@@ -2023,7 +2062,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>67</v>
       </c>
@@ -2099,7 +2138,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>75</v>
       </c>
@@ -2177,7 +2216,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>84</v>
       </c>
@@ -2253,7 +2292,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>93</v>
       </c>
@@ -2329,7 +2368,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>102</v>
       </c>
@@ -2405,7 +2444,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>111</v>
       </c>
@@ -2481,7 +2520,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>121</v>
       </c>
@@ -2504,318 +2543,382 @@
       <c r="H15" s="3">
         <v>4</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="3"/>
+      <c r="I15" s="3">
+        <v>4</v>
+      </c>
+      <c r="J15" s="3">
+        <v>3</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="L15" s="3">
+        <v>450</v>
+      </c>
       <c r="M15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="R15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="T15" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V15" s="4"/>
+      <c r="V15" s="5" t="s">
+        <v>127</v>
+      </c>
       <c r="W15" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="X15" s="4"/>
+        <v>128</v>
+      </c>
+      <c r="X15" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y15" s="7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B16" s="3">
         <v>3</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H16" s="3">
         <v>32</v>
       </c>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="3"/>
+      <c r="I16" s="3">
+        <v>23</v>
+      </c>
+      <c r="J16" s="3">
+        <v>20</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="L16" s="3">
+        <v>200</v>
+      </c>
       <c r="M16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="R16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="S16" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="T16" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U16" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V16" s="4"/>
+      <c r="V16" s="5" t="s">
+        <v>136</v>
+      </c>
       <c r="W16" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="X16" s="4"/>
+        <v>137</v>
+      </c>
+      <c r="X16" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y16" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="17" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B17" s="3">
         <v>3</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="H17" s="3">
         <v>15</v>
       </c>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="3"/>
+      <c r="I17" s="3">
+        <v>15</v>
+      </c>
+      <c r="J17" s="3">
+        <v>15</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="L17" s="3">
+        <v>40</v>
+      </c>
       <c r="M17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="R17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="S17" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="T17" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U17" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V17" s="4"/>
+      <c r="V17" s="5" t="s">
+        <v>145</v>
+      </c>
       <c r="W17" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="X17" s="4"/>
-      <c r="Y17" s="7"/>
-    </row>
-    <row r="18" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+      <c r="X17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H18" s="3">
         <v>8</v>
       </c>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="3"/>
+      <c r="I18" s="3">
+        <v>8</v>
+      </c>
+      <c r="J18" s="3">
+        <v>8</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="L18" s="3">
+        <v>150</v>
+      </c>
       <c r="M18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="R18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="S18" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="T18" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U18" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V18" s="4"/>
+      <c r="V18" s="5" t="s">
+        <v>154</v>
+      </c>
       <c r="W18" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="7"/>
-    </row>
-    <row r="19" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="X18" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y18" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="B19" s="3">
         <v>3</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="H19" s="3">
         <v>3</v>
       </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="3"/>
+      <c r="I19" s="3">
+        <v>3</v>
+      </c>
+      <c r="J19" s="3">
+        <v>3</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="L19" s="3">
+        <v>50</v>
+      </c>
       <c r="M19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="R19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="S19" s="3" t="s">
-        <v>126</v>
+        <v>33</v>
       </c>
       <c r="T19" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U19" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V19" s="4"/>
+      <c r="V19" s="5" t="s">
+        <v>163</v>
+      </c>
       <c r="W19" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="X19" s="4"/>
+        <v>164</v>
+      </c>
+      <c r="X19" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y19" s="7" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="B20" s="3">
         <v>4</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="H20" s="3">
         <v>7</v>
@@ -2825,25 +2928,25 @@
       <c r="K20" s="4"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2854,30 +2957,30 @@
       </c>
       <c r="V20" s="4"/>
       <c r="W20" s="4" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="X20" s="4"/>
       <c r="Y20" s="7"/>
     </row>
     <row r="21" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B21" s="3">
         <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="H21" s="3">
         <v>11</v>
@@ -2887,25 +2990,25 @@
       <c r="K21" s="4"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T21" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2916,30 +3019,30 @@
       </c>
       <c r="V21" s="4"/>
       <c r="W21" s="4" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="X21" s="4"/>
       <c r="Y21" s="7"/>
     </row>
     <row r="22" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B22" s="3">
         <v>4</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="H22" s="3">
         <v>24</v>
@@ -2949,25 +3052,25 @@
       <c r="K22" s="4"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T22" s="6" t="str">
         <f t="shared" si="0"/>
@@ -2978,32 +3081,32 @@
       </c>
       <c r="V22" s="4"/>
       <c r="W22" s="4" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="X22" s="4"/>
       <c r="Y22" s="7"/>
     </row>
     <row r="23" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B23" s="3">
         <v>4</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="H23" s="3">
         <v>4</v>
@@ -3013,25 +3116,25 @@
       <c r="K23" s="4"/>
       <c r="L23" s="3"/>
       <c r="M23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T23" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3042,34 +3145,34 @@
       </c>
       <c r="V23" s="4"/>
       <c r="W23" s="4" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="X23" s="4"/>
       <c r="Y23" s="7" t="s">
-        <v>128</v>
+        <v>192</v>
       </c>
     </row>
     <row r="24" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="B24" s="3">
         <v>4</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="H24" s="3">
         <v>12</v>
@@ -3079,25 +3182,25 @@
       <c r="K24" s="4"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T24" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3108,32 +3211,32 @@
       </c>
       <c r="V24" s="4"/>
       <c r="W24" s="4" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="X24" s="4"/>
       <c r="Y24" s="7"/>
     </row>
     <row r="25" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="B25" s="3">
         <v>5</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="H25" s="3">
         <v>5</v>
@@ -3143,25 +3246,25 @@
       <c r="K25" s="4"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3172,34 +3275,34 @@
       </c>
       <c r="V25" s="4"/>
       <c r="W25" s="4" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="7" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="26" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="B26" s="3">
         <v>5</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="H26" s="3">
         <v>94</v>
@@ -3209,25 +3312,25 @@
       <c r="K26" s="4"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3238,32 +3341,32 @@
       </c>
       <c r="V26" s="4"/>
       <c r="W26" s="4" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="X26" s="4"/>
       <c r="Y26" s="7"/>
     </row>
-    <row r="27" spans="1:25" ht="51" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="B27" s="3">
         <v>0</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="H27" s="3">
         <v>161</v>
@@ -3275,7 +3378,7 @@
         <v>148</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="L27" s="3">
         <v>1100</v>
@@ -3309,39 +3412,39 @@
         <v>34</v>
       </c>
       <c r="V27" s="5" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="W27" s="4" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="X27" s="4" t="s">
         <v>37</v>
       </c>
       <c r="Y27" s="7" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="B28" s="3">
         <v>5</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="H28" s="3">
         <v>67</v>
@@ -3351,25 +3454,25 @@
       <c r="K28" s="4"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3380,32 +3483,32 @@
       </c>
       <c r="V28" s="4"/>
       <c r="W28" s="4" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="X28" s="4"/>
       <c r="Y28" s="7"/>
     </row>
     <row r="29" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="B29" s="3">
         <v>5</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="H29" s="3">
         <v>31</v>
@@ -3415,25 +3518,25 @@
       <c r="K29" s="4"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T29" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3444,30 +3547,30 @@
       </c>
       <c r="V29" s="4"/>
       <c r="W29" s="4" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="X29" s="4"/>
       <c r="Y29" s="7"/>
     </row>
     <row r="30" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="B30" s="3">
         <v>5</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="H30" s="3">
         <v>5</v>
@@ -3477,25 +3580,25 @@
       <c r="K30" s="4"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T30" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3506,32 +3609,32 @@
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="4" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="7" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="31" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="B31" s="3">
         <v>6</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="H31" s="3">
         <v>1</v>
@@ -3541,25 +3644,25 @@
       <c r="K31" s="4"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T31" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3570,32 +3673,32 @@
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="4" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="7" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="H32" s="3">
         <v>2</v>
@@ -3605,25 +3708,25 @@
       <c r="K32" s="4"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T32" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3634,32 +3737,32 @@
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="4" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="7" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="33" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="B33" s="3">
         <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="H33" s="3">
         <v>2</v>
@@ -3669,25 +3772,25 @@
       <c r="K33" s="4"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3698,34 +3801,34 @@
       </c>
       <c r="V33" s="4"/>
       <c r="W33" s="4" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="X33" s="4"/>
       <c r="Y33" s="7" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="34" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="B34" s="3">
         <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H34" s="3">
         <v>8</v>
@@ -3735,25 +3838,25 @@
       <c r="K34" s="4"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3764,32 +3867,32 @@
       </c>
       <c r="V34" s="4"/>
       <c r="W34" s="4" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="X34" s="4"/>
       <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="B35" s="3">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="H35" s="3">
         <v>14</v>
@@ -3799,25 +3902,25 @@
       <c r="K35" s="4"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T35" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3828,32 +3931,32 @@
       </c>
       <c r="V35" s="4"/>
       <c r="W35" s="4" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="X35" s="4"/>
       <c r="Y35" s="7"/>
     </row>
     <row r="36" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="B36" s="3">
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="H36" s="3">
         <v>1</v>
@@ -3863,25 +3966,25 @@
       <c r="K36" s="4"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3892,34 +3995,34 @@
       </c>
       <c r="V36" s="4"/>
       <c r="W36" s="4" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="X36" s="4"/>
       <c r="Y36" s="7" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
     </row>
     <row r="37" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="B37" s="3">
         <v>7</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
@@ -3929,25 +4032,25 @@
       <c r="K37" s="4"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3958,34 +4061,34 @@
       </c>
       <c r="V37" s="4"/>
       <c r="W37" s="4" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="X37" s="4"/>
       <c r="Y37" s="7" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="B38" s="3">
         <v>7</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="H38" s="3">
         <v>2</v>
@@ -3995,25 +4098,25 @@
       <c r="K38" s="4"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4024,34 +4127,34 @@
       </c>
       <c r="V38" s="4"/>
       <c r="W38" s="4" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="X38" s="4"/>
       <c r="Y38" s="7" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="B39" s="3">
         <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="H39" s="3">
         <v>6</v>
@@ -4061,25 +4164,25 @@
       <c r="K39" s="4"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4090,32 +4193,32 @@
       </c>
       <c r="V39" s="4"/>
       <c r="W39" s="4" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="X39" s="4"/>
       <c r="Y39" s="7"/>
     </row>
     <row r="40" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="B40" s="3">
         <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="H40" s="3">
         <v>33</v>
@@ -4125,25 +4228,25 @@
       <c r="K40" s="4"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T40" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4154,32 +4257,32 @@
       </c>
       <c r="V40" s="4"/>
       <c r="W40" s="4" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="X40" s="4"/>
       <c r="Y40" s="7" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
     </row>
     <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="B41" s="3">
         <v>8</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="H41" s="3">
         <v>9</v>
@@ -4189,25 +4292,25 @@
       <c r="K41" s="4"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4218,30 +4321,30 @@
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="X41" s="4"/>
       <c r="Y41" s="7"/>
     </row>
     <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
@@ -4251,25 +4354,25 @@
       <c r="K42" s="4"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4280,32 +4383,32 @@
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="X42" s="4"/>
       <c r="Y42" s="7" t="s">
-        <v>128</v>
+        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
@@ -4315,25 +4418,25 @@
       <c r="K43" s="4"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4344,32 +4447,32 @@
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="X43" s="4"/>
       <c r="Y43" s="7" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>314</v>
+        <v>327</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>315</v>
+        <v>328</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
@@ -4379,25 +4482,25 @@
       <c r="K44" s="4"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4408,11 +4511,11 @@
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="X44" s="4"/>
       <c r="Y44" s="7" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -4492,65 +4595,70 @@
     <hyperlink ref="V14" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
     <hyperlink ref="F15" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
     <hyperlink ref="G15" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="F16" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="G16" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="F17" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="G17" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="F18" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="G18" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="F19" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="G19" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="F20" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="G20" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="F21" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="G21" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="F22" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="G22" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="F23" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="G23" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="F24" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="G24" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="F25" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="G25" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="F26" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="G26" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="F27" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="G27" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="V27" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="F28" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="G28" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="F29" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="G29" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="F30" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="G30" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="F31" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="G31" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="F32" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="G32" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="F33" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="G33" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="F34" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="G34" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="F35" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="G35" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="F36" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="G36" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="F37" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="G37" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="F38" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="G38" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="F39" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="G39" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="F40" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="G40" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="F41" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="G41" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="F42" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="G42" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="F43" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="G43" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="F44" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="G44" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="V15" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="F16" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="G16" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="V16" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="F17" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="G17" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="V17" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="F18" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="G18" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="V18" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="F19" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="G19" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="V19" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="F20" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="G20" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="F21" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="G21" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="F22" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="G22" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="F23" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="G23" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="F24" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="G24" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="F25" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="G25" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="F26" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="G26" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="F27" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="G27" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="V27" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="F28" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="G28" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="F29" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="G29" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="F30" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="G30" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="F31" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="G31" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="F32" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="G32" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="F33" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="G33" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="F34" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="G34" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="F35" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="G35" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="F36" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="G36" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="F37" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="G37" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="F38" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="G38" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="F39" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="G39" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="F40" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="G40" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="F41" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="G41" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="F42" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="G42" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="F43" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="G43" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="F44" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="G44" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4570,25 +4678,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -4597,16 +4705,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -4615,16 +4723,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -4633,7 +4741,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -4642,7 +4750,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -4651,27 +4759,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>342</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4680,11 +4788,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -4693,11 +4801,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -4706,11 +4814,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4719,11 +4827,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -4732,11 +4840,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -4745,11 +4853,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -4758,16 +4866,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.27500000000000002</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -4775,16 +4883,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -4860,7 +4968,7 @@
       </c>
       <c r="C29" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A29,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D29" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A29,Pages!$U$5:$U$44,"Approved")</f>
@@ -4868,7 +4976,7 @@
       </c>
       <c r="E29" s="6" t="str">
         <f>IF(D29=B29,"Approved",IF(C29=B29,"Ready for client review",IF(C29&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A29,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -4992,15 +5100,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5008,7 +5116,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -5016,7 +5124,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -5024,7 +5132,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5032,7 +5140,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -5040,7 +5148,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5048,7 +5156,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -5056,7 +5164,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5064,28 +5172,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Tracker: batch 4 (P16-19b) ready for client review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67B4A47-6B94-4D9D-A200-2DC5B1B85C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A55A780-B555-4C03-AF81-02F95ADEDFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="379">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -154,7 +154,7 @@
     <t>2026-10-02</t>
   </si>
   <si>
-    <t>Built. Only 5 units, all process-scale (Carr Centritech Centritec Cell 8, Sharples Type 1P, a beaker centrifuge), not benchtop instruments; the copy says so. 'lab centrifuge' and 'ultracentrifuge' demand is lab-instrument (Beckman, Thermo), so the ultracentrifuge terms are excluded. No size or condition tabs (all used). 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built. Only 5 units, all process-scale (Carr Centritech Centritec Cell 8, Sharples Type 1P, a beaker centrifuge), not benchtop instruments; the copy says so. 'lab centrifuge' and 'ultracentrifuge' demand is lab-instrument (Beckman, Thermo), so the ultracentrifuge terms are excluded. No size or condition tabs (all used). 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>2</t>
@@ -181,7 +181,7 @@
     <t>equipment/centrifuge/misc-and-hydraulic-centrifuge/INTERNAL-REVIEW-misc-and-hydraulic-centrifuge.html</t>
   </si>
   <si>
-    <t>Built as 'Tubular, Podbielniak &amp; Hydraulic Centrifuges': IMS's misc bucket is Sharples tubular super centrifuges, Podbielniak extractors and hydraulic drives. 'Hydraulic centrifuge' has no search demand; the page targets tubular / super / sharples / centrifugal extractor. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built as 'Tubular, Podbielniak &amp; Hydraulic Centrifuges': IMS's misc bucket is Sharples tubular super centrifuges, Podbielniak extractors and hydraulic drives. 'Hydraulic centrifuge' has no search demand; the page targets tubular / super / sharples / centrifugal extractor. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>3</t>
@@ -208,7 +208,7 @@
     <t>equipment/centrifuge/peeler-centrifuge/INTERNAL-REVIEW-peeler-centrifuge.html</t>
   </si>
   <si>
-    <t>Built. IPP's blog already ranks for 'what is a peeler centrifuge' and 'peeler vs pusher', so the FAQ answers briefly and links to those guides. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built. IPP's blog already ranks for 'what is a peeler centrifuge' and 'peeler vs pusher', so the FAQ answers briefly and links to those guides. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>4</t>
@@ -238,7 +238,7 @@
     <t>equipment/centrifuge/pusher-centrifuge-parts/INTERNAL-REVIEW-pusher-centrifuge-parts.html</t>
   </si>
   <si>
-    <t>Built. 21 parts listings, only 1 with a photo, mostly Krauss Maffei SB1000/2 components. Part type comes from the IMS description, and browse cards use IMS keyword search. Generic 'centrifuge parts' demand is lab-instrument parts, so it is excluded. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built. 21 parts listings, only 1 with a photo, mostly Krauss Maffei SB1000/2 components. Part type comes from the IMS description, and browse cards use IMS keyword search. Generic 'centrifuge parts' demand is lab-instrument parts, so it is excluded. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>5</t>
@@ -262,7 +262,7 @@
     <t>equipment/centrifuge/pusher-centrifuge/INTERNAL-REVIEW-pusher-centrifuge.html</t>
   </si>
   <si>
-    <t>Built from 26 complete machines (the 21 parts-only listings are on priority 4). The IMS 'Browse All' links show IMS's own pusher search, which includes the parts. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built from 26 complete machines (the 21 parts-only listings are on priority 4). The IMS 'Browse All' links show IMS's own pusher search, which includes the parts. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>6</t>
@@ -289,7 +289,7 @@
     <t>equipment/centrifuge/solid-bowl-decanter-centrifuge-parts/INTERNAL-REVIEW-solid-bowl-decanter-centrifuge-parts.html</t>
   </si>
   <si>
-    <t>Built. 7 parts listings, all with photos: scroll conveyors (Sharples P3400, Alfa Laval NX314, Dorr Oliver for the 16L and Z3L), Sharples P-2000 and Sangerhausen rotating assemblies, and a Bird gearbox. Part type comes from the IMS description. Complete-machine and repair queries are excluded (the live decanter page owns machines). Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built. 7 parts listings, all with photos: scroll conveyors (Sharples P3400, Alfa Laval NX314, Dorr Oliver for the 16L and Z3L), Sharples P-2000 and Sangerhausen rotating assemblies, and a Bird gearbox. Part type comes from the IMS description. Complete-machine and repair queries are excluded (the live decanter page owns machines). Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>7</t>
@@ -316,7 +316,7 @@
     <t>equipment/dryer/nauta-dryer/INTERNAL-REVIEW-nauta-dryer.html</t>
   </si>
   <si>
-    <t>Built. 11 units from 9 OEMs (Krauss Maffei, Bolz, Vrieco Nauta, Hosokawa Alpine and others). Nauta mixer terms are excluded (the live Nauta mixer page owns them); double cone terms belong to the twin shell page, linked from the comparison table. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built. 11 units from 9 OEMs (Krauss Maffei, Bolz, Vrieco Nauta, Hosokawa Alpine and others). Nauta mixer terms are excluded (the live Nauta mixer page owns them); double cone terms belong to the twin shell page, linked from the comparison table. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>8</t>
@@ -343,7 +343,7 @@
     <t>equipment/dryer/drum-dryer/INTERNAL-REVIEW-drum-dryer.html</t>
   </si>
   <si>
-    <t>Built. 16 listings: Simon Dryers, Blaw Knox and Gouda single and double drum dryers plus unused spare drums. Household laundry dryer and rotary drum dryer terms are excluded. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built. 16 listings: Simon Dryers, Blaw Knox and Gouda single and double drum dryers plus unused spare drums. Household laundry dryer and rotary drum dryer terms are excluded. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>9</t>
@@ -370,7 +370,7 @@
     <t>equipment/dryer/flash-dryer/INTERNAL-REVIEW-flash-dryer.html</t>
   </si>
   <si>
-    <t>Built (new URL, no live page). Only 4 units: APV Anhydro spin flash, Aljet, Hosokawa Alpine MDV-4, AKSH Engineering. Screen-printing flash dryers dominate 'flash dryer' demand, so the H1 says industrial. The IMS inlet-moisture fields and the Hosokawa evaporation field are mislabelled, so they are not published. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built (new URL, no live page). Only 4 units: APV Anhydro spin flash, Aljet, Hosokawa Alpine MDV-4, AKSH Engineering. Screen-printing flash dryers dominate 'flash dryer' demand, so the H1 says industrial. The IMS inlet-moisture fields and the Hosokawa evaporation field are mislabelled, so they are not published. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>10</t>
@@ -400,7 +400,7 @@
     <t>equipment/dryer/porcupine-dryer-parts/INTERNAL-REVIEW-porcupine-dryer-parts.html</t>
   </si>
   <si>
-    <t>Built (new URL). 4 GPS listings: 3 troughs and a new shaft and flights set. 'porcupine dryer' demand belongs to the live porcupine dryer page, linked from an FAQ. Parts queries have no measured volume. The GPS/Bethlehem brand angle comes from IPP's own news post (not linked). Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
+    <t>Built (new URL). 4 GPS listings: 3 troughs and a new shaft and flights set. 'porcupine dryer' demand belongs to the live porcupine dryer page, linked from an FAQ. Parts queries have no measured volume. The GPS/Bethlehem brand angle comes from IPP's own news post (not linked). Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>11</t>
@@ -427,7 +427,7 @@
     <t>equipment/dryer/rotary-hot-air-dryer/INTERNAL-REVIEW-rotary-hot-air-dryer.html</t>
   </si>
   <si>
-    <t>Built from 4 units: a Standard Steel louver dryer and a Patterson Kelly unit in stainless steel 304, a Link Belt in carbon steel, and a refurbished stainless steel 316 co-current dryer. The refurbished listing says both 'direct fired' and steam; the copy uses steam. Comparison links to the live rotary steam tube dryer page. Manufacturer, design, maintenance, triple-pass and household vent terms excluded.</t>
+    <t>Built from 4 units: a Standard Steel louver dryer and a Patterson Kelly unit in stainless steel 304, a Link Belt in carbon steel, and a refurbished stainless steel 316 co-current dryer. The refurbished listing says both 'direct fired' and steam; the copy uses steam. Comparison links to the live rotary steam tube dryer page. Manufacturer, design, maintenance, triple-pass and household vent terms excluded. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>12</t>
@@ -454,7 +454,7 @@
     <t>equipment/dryer/shelf-dryer/INTERNAL-REVIEW-shelf-dryer.html</t>
   </si>
   <si>
-    <t>Built from 23 listings: 22 good used vacuum shelf and tray dryers and a new GPS vacuum tray dryer. The IMS shelf-dryer search also returns oven dryers; they stay off the page. The Stokes hot water generator is described as an accessory. Unit defect notes and mis-entered IMS dimensions are not repeated. The IMS Leybold manufacturer filter is broken (returns all 32), so Leybold has no tab. Pharmaceutical, rotary tray, household and parts terms excluded.</t>
+    <t>Built from 23 listings: 22 good used vacuum shelf and tray dryers and a new GPS vacuum tray dryer. The IMS shelf-dryer search also returns oven dryers; they stay off the page. The Stokes hot water generator is described as an accessory. Unit defect notes and mis-entered IMS dimensions are not repeated. The IMS Leybold manufacturer filter is broken (returns all 32), so Leybold has no tab. Pharmaceutical, rotary tray, household and parts terms excluded. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>13</t>
@@ -481,7 +481,7 @@
     <t>equipment/dryer/thin-film-dryer/INTERNAL-REVIEW-thin-film-dryer.html</t>
   </si>
   <si>
-    <t>Built from 15 units: Luwa SMS DK600, D-850 and 1000/6000 dryers and a Buss-SMS-Canzler D-015, all stainless. IMS lists the DK600 units as coolers; an FAQ covers cooling duty. Thin film evaporator terms are excluded (IPP's evaporator page and blog own them); the comparison links to the live evaporator page.</t>
+    <t>Built from 15 units: Luwa SMS DK600, D-850 and 1000/6000 dryers and a Buss-SMS-Canzler D-015, all stainless. IMS lists the DK600 units as coolers; an FAQ covers cooling duty. Thin film evaporator terms are excluded (IPP's evaporator page and blog own them); the comparison links to the live evaporator page. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>14</t>
@@ -508,7 +508,7 @@
     <t>equipment/dryer/thermal-disc-dryer/INTERNAL-REVIEW-thermal-disc-dryer.html</t>
   </si>
   <si>
-    <t>Built from 8 units: unused surplus Bepex TorusDisc TD48-9 units, a Bepex Model 60-14, a Bethlehem processor and a Strong Scott TDJ. IMS lists the TD48-9 units as coolers; unit 239472 has no IMS data. Comparison links to the live porcupine dryer page. Sludge, rendering and fish meal (application) terms excluded.</t>
+    <t>Built from 8 units: unused surplus Bepex TorusDisc TD48-9 units, a Bepex Model 60-14, a Bethlehem processor and a Strong Scott TDJ. IMS lists the TD48-9 units as coolers; unit 239472 has no IMS data. Comparison links to the live porcupine dryer page. Sludge, rendering and fish meal (application) terms excluded. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>15</t>
@@ -535,7 +535,7 @@
     <t>equipment/dryer/spherical-dryer/INTERNAL-REVIEW-spherical-dryer.html</t>
   </si>
   <si>
-    <t>Built from 3 units: two Rosenmund AG RKT-2000 dryers and a Pierre Guerin Turbosphere TS200, jacketed, stainless steel 316L. Rosenmund vessel and jacket pressures are not published (the IMS fields look swapped or inconsistent) and the IMS model field holds the town. The comparison links to the Nauta dryer page, which is new and not live yet, so publish them together.</t>
+    <t>Built from 3 units: two Rosenmund AG RKT-2000 dryers and a Pierre Guerin Turbosphere TS200, jacketed, stainless steel 316L. Rosenmund vessel and jacket pressures are not published (the IMS fields look swapped or inconsistent) and the IMS model field holds the town. The comparison links to the Nauta dryer page, which is new and not live yet, so publish them together. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
   </si>
   <si>
     <t>16</t>
@@ -553,442 +553,487 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/pan-dryer</t>
   </si>
   <si>
+    <t>pan dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/pan-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/pan-dryer/INTERNAL-REVIEW-pan-dryer.html</t>
+  </si>
+  <si>
+    <t>Built from 7 units: Buflovak/Blaw Knox Grainer pans (no photos on IMS), a Guedu 3500, a Bonazzi Mario 881 LT 1000 and an unbranded stainless steel 304 pan. Only design capacity is published: two listings give a working capacity above it. No listing names an agitator, so agitation is described as the design type only. Comparison links to the live rotary vacuum dryer page.</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Dryer-Oven</t>
+  </si>
+  <si>
+    <t>Oven Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/oven-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/oven-dryer</t>
+  </si>
+  <si>
+    <t>drying oven</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/oven-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/oven-dryer/INTERNAL-REVIEW-oven-dryer.html</t>
+  </si>
+  <si>
+    <t>Built as 'Industrial Drying Ovens' from 11 units: Hedinair and Lewco drum warming ovens, Amarc drum and IBC ovens, Barlow Whitney vacuum ovens, a Lytzen shelf oven, a Caltherm two-chamber oven and Normandie-Labo and Better Built lab ovens. The Caltherm's -16.7 C rating is an IMS error and stays off the page. The comparison links to the shelf dryer page (new URL, publish together). Lab-instrument brands and drum heater blankets are excluded.</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>Dryer-Flaker Drum and Belt</t>
+  </si>
+  <si>
+    <t>Flaker Drum and Belt Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/flaker-drum-and-belt-dryer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/flaker-drum-and-belt-dryer</t>
+  </si>
+  <si>
+    <t>drum flaker</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/flaker-drum-and-belt-dryer/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/flaker-drum-and-belt-dryer/INTERNAL-REVIEW-flaker-drum-and-belt-dryer.html</t>
+  </si>
+  <si>
+    <t>Built as 'Drum &amp; Belt Flakers' from 24 listings: belt flakers and pastillators (Sandvik, Berndorf, Kaiser, Steel Belt Systems and others) and drum flakers (Simon Dryers, APV Mitchell, Blaw Knox, Gouda and others), plus two spare drums. First page with drum/belt type tabs. Three mis-entered IMS areas or widths (Simon 228 m2, APV 28 mm and 26 m2, MBT 4 m2) are kept off the cards. IMS has no drum filter, so the drum tab links to the whole category. The FAQ links the drum dryer page (new URL). Ice flakers, grain flaking mills and Jayden Flaker are excluded.</t>
+  </si>
+  <si>
+    <t>19a</t>
+  </si>
+  <si>
+    <t>Dryer-Air</t>
+  </si>
+  <si>
+    <t>Desiccant</t>
+  </si>
+  <si>
+    <t>Desiccant Air Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/desiccant/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/air-dryer/desiccant</t>
+  </si>
+  <si>
+    <t>desiccant air dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/desiccant/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/desiccant/INTERNAL-REVIEW-desiccant.html</t>
+  </si>
+  <si>
+    <t>Built from 4 listings: PneumaTech PE-3100, Arrow RH212A heatless, a Sullair self-recharging dryer and one listing with no data. Dew points and purge figures come from the SERP evidence (Sullair, Atlas Copco). The comparison links the refrigerated page (new URL, publish together). Plastic resin dryers, rentals and inline cartridges are excluded.</t>
+  </si>
+  <si>
+    <t>19b</t>
+  </si>
+  <si>
+    <t>Refrigerant/Heat</t>
+  </si>
+  <si>
+    <t>Refrigerated Air Dryers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/dryer/refrigerant-heat/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/air-dryer/refrigerant-heat</t>
+  </si>
+  <si>
+    <t>refrigerated air dryer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/dryer/refrigerant-heat/</t>
+  </si>
+  <si>
+    <t>equipment/dryer/refrigerant-heat/INTERNAL-REVIEW-refrigerant-heat.html</t>
+  </si>
+  <si>
+    <t>Built from 12 listings: Atlas Copco FD units, Hankinson 801600, Ingersoll Rand DXR 2000W and TS 2000, M.T.A DE235 HP and a 1000DES/HYD. The IMS category also holds an Atlas Copco CD335+ (a desiccant model, named without a type), an Oriad electric dryer and natural gas air heater skids. The IMS Ingersoll Rand filter returns the whole category, so it has no tab. The FAQ links the desiccant page (new URL).</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Heat Exchanger</t>
+  </si>
+  <si>
+    <t>Air Fin</t>
+  </si>
+  <si>
+    <t>Air Fin Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/air-fin/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/air-fin</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>equipment/dryer/pan-dryer/INTERNAL-REVIEW-pan-dryer.html</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>Dryer-Oven</t>
-  </si>
-  <si>
-    <t>Oven Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/oven-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/oven-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/oven-dryer/INTERNAL-REVIEW-oven-dryer.html</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>Dryer-Flaker Drum and Belt</t>
-  </si>
-  <si>
-    <t>Flaker Drum and Belt Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/flaker-drum-and-belt-dryer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/flaker-drum-and-belt-dryer</t>
-  </si>
-  <si>
-    <t>equipment/dryer/flaker-drum-and-belt-dryer/INTERNAL-REVIEW-flaker-drum-and-belt-dryer.html</t>
-  </si>
-  <si>
-    <t>19a</t>
-  </si>
-  <si>
-    <t>Dryer-Air</t>
-  </si>
-  <si>
-    <t>Desiccant</t>
-  </si>
-  <si>
-    <t>Desiccant Air Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/desiccant/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/air-dryer/desiccant</t>
-  </si>
-  <si>
-    <t>equipment/dryer/desiccant/INTERNAL-REVIEW-desiccant.html</t>
+    <t>equipment/heat-exchanger/air-fin/INTERNAL-REVIEW-air-fin.html</t>
+  </si>
+  <si>
+    <t>Thin inventory: 5 units.</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>Block</t>
+  </si>
+  <si>
+    <t>Block Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/block/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/block</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/block/INTERNAL-REVIEW-block.html</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Plate and Frame</t>
+  </si>
+  <si>
+    <t>Plate and Frame Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/plate-and-frame/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/plate-and-frame</t>
+  </si>
+  <si>
+    <t>plate and frame heat exchanger</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/plate-and-frame/</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/plate-and-frame/INTERNAL-REVIEW-plate-and-frame.html</t>
+  </si>
+  <si>
+    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Spiral</t>
+  </si>
+  <si>
+    <t>Spiral Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/spiral/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/spiral</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/spiral/INTERNAL-REVIEW-spiral.html</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>Welded Plate</t>
+  </si>
+  <si>
+    <t>Welded Plate Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/welded-plate/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/welded-plate</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/welded-plate/INTERNAL-REVIEW-welded-plate.html</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Homogenizer</t>
+  </si>
+  <si>
+    <t>Homogenizers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/homogenizer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/homogenizer</t>
+  </si>
+  <si>
+    <t>equipment/homogenizer/INTERNAL-REVIEW-homogenizer.html</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Incinerator</t>
+  </si>
+  <si>
+    <t>Incinerators</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/incinerator/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/incinerator</t>
+  </si>
+  <si>
+    <t>equipment/incinerator/INTERNAL-REVIEW-incinerator.html</t>
+  </si>
+  <si>
+    <t>Thin inventory: 1 unit on IMS.</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>Kettle</t>
+  </si>
+  <si>
+    <t>Kettles</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/kettle/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kettle</t>
+  </si>
+  <si>
+    <t>equipment/kettle/INTERNAL-REVIEW-kettle.html</t>
+  </si>
+  <si>
+    <t>Thin inventory: 2 units.</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Kiln</t>
+  </si>
+  <si>
+    <t>Kilns</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/kiln/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kiln</t>
+  </si>
+  <si>
+    <t>equipment/kiln/INTERNAL-REVIEW-kiln.html</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>Mill</t>
+  </si>
+  <si>
+    <t>Ball</t>
+  </si>
+  <si>
+    <t>Ball Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/ball/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/ball</t>
+  </si>
+  <si>
+    <t>equipment/mill/ball/INTERNAL-REVIEW-ball.html</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Colloid</t>
+  </si>
+  <si>
+    <t>Colloid Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/colloid/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/colloid</t>
+  </si>
+  <si>
+    <t>equipment/mill/colloid/INTERNAL-REVIEW-colloid.html</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Kady</t>
+  </si>
+  <si>
+    <t>Kady Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/kady/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/kady</t>
+  </si>
+  <si>
+    <t>equipment/mill/kady/INTERNAL-REVIEW-kady.html</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>Pebble</t>
+  </si>
+  <si>
+    <t>Pebble Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/pebble/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pebble</t>
+  </si>
+  <si>
+    <t>equipment/mill/pebble/INTERNAL-REVIEW-pebble.html</t>
+  </si>
+  <si>
+    <t>IMS shows 0 units. The page will be a sourcing page with no listing.</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Pellet</t>
+  </si>
+  <si>
+    <t>Pellet Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/pellet/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pellet</t>
+  </si>
+  <si>
+    <t>equipment/mill/pellet/INTERNAL-REVIEW-pellet.html</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>Roll</t>
+  </si>
+  <si>
+    <t>Roll Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/roll/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/roll</t>
+  </si>
+  <si>
+    <t>equipment/mill/roll/INTERNAL-REVIEW-roll.html</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>Shot And Sand</t>
+  </si>
+  <si>
+    <t>Shot and Sand Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/shot-and-sand/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/shot-and-sand</t>
+  </si>
+  <si>
+    <t>equipment/mill/shot-and-sand/INTERNAL-REVIEW-shot-and-sand.html</t>
+  </si>
+  <si>
+    <t>IMS Mill &gt; Shot And Sand (33 listings). IMS also has a separate Mixer-Shot and Sand type, so check the entity overlap.</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>Mixer-Banbury</t>
+  </si>
+  <si>
+    <t>Banbury Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/banbury-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/banbury-mixer</t>
+  </si>
+  <si>
+    <t>equipment/mixer/banbury-mixer/INTERNAL-REVIEW-banbury-mixer.html</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>Mixer-Charge Can and Pony</t>
+  </si>
+  <si>
+    <t>Charge Can and Pony Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/charge-can-and-pony-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/charge-can-and-pony-mixer</t>
+  </si>
+  <si>
+    <t>equipment/mixer/charge-can-and-pony-mixer/INTERNAL-REVIEW-charge-can-and-pony-mixer.html</t>
   </si>
   <si>
     <t>Thin inventory: 4 units.</t>
-  </si>
-  <si>
-    <t>19b</t>
-  </si>
-  <si>
-    <t>Refrigerant/Heat</t>
-  </si>
-  <si>
-    <t>Refrigerated Air Dryers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/dryer/refrigerant-heat/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/air-dryer/refrigerant-heat</t>
-  </si>
-  <si>
-    <t>equipment/dryer/refrigerant-heat/INTERNAL-REVIEW-refrigerant-heat.html</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>Heat Exchanger</t>
-  </si>
-  <si>
-    <t>Air Fin</t>
-  </si>
-  <si>
-    <t>Air Fin Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/air-fin/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/air-fin</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/air-fin/INTERNAL-REVIEW-air-fin.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 5 units.</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>Block</t>
-  </si>
-  <si>
-    <t>Block Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/block/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/block</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/block/INTERNAL-REVIEW-block.html</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>Plate and Frame</t>
-  </si>
-  <si>
-    <t>Plate and Frame Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/plate-and-frame/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/plate-and-frame</t>
-  </si>
-  <si>
-    <t>plate and frame heat exchanger</t>
-  </si>
-  <si>
-    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/plate-and-frame/</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/plate-and-frame/INTERNAL-REVIEW-plate-and-frame.html</t>
-  </si>
-  <si>
-    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued.</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>Spiral</t>
-  </si>
-  <si>
-    <t>Spiral Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/spiral/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/spiral</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/spiral/INTERNAL-REVIEW-spiral.html</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>Welded Plate</t>
-  </si>
-  <si>
-    <t>Welded Plate Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/welded-plate/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/welded-plate</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/welded-plate/INTERNAL-REVIEW-welded-plate.html</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>Homogenizer</t>
-  </si>
-  <si>
-    <t>Homogenizers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/homogenizer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/homogenizer</t>
-  </si>
-  <si>
-    <t>equipment/homogenizer/INTERNAL-REVIEW-homogenizer.html</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>Incinerator</t>
-  </si>
-  <si>
-    <t>Incinerators</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/incinerator/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/incinerator</t>
-  </si>
-  <si>
-    <t>equipment/incinerator/INTERNAL-REVIEW-incinerator.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 1 unit on IMS.</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>Kettle</t>
-  </si>
-  <si>
-    <t>Kettles</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/kettle/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kettle</t>
-  </si>
-  <si>
-    <t>equipment/kettle/INTERNAL-REVIEW-kettle.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 2 units.</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>Kiln</t>
-  </si>
-  <si>
-    <t>Kilns</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/kiln/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kiln</t>
-  </si>
-  <si>
-    <t>equipment/kiln/INTERNAL-REVIEW-kiln.html</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>Mill</t>
-  </si>
-  <si>
-    <t>Ball</t>
-  </si>
-  <si>
-    <t>Ball Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/ball/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/ball</t>
-  </si>
-  <si>
-    <t>equipment/mill/ball/INTERNAL-REVIEW-ball.html</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Colloid</t>
-  </si>
-  <si>
-    <t>Colloid Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/colloid/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/colloid</t>
-  </si>
-  <si>
-    <t>equipment/mill/colloid/INTERNAL-REVIEW-colloid.html</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>Kady</t>
-  </si>
-  <si>
-    <t>Kady Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/kady/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/kady</t>
-  </si>
-  <si>
-    <t>equipment/mill/kady/INTERNAL-REVIEW-kady.html</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>Pebble</t>
-  </si>
-  <si>
-    <t>Pebble Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/pebble/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pebble</t>
-  </si>
-  <si>
-    <t>equipment/mill/pebble/INTERNAL-REVIEW-pebble.html</t>
-  </si>
-  <si>
-    <t>IMS shows 0 units. The page will be a sourcing page with no listing.</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>Pellet</t>
-  </si>
-  <si>
-    <t>Pellet Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/pellet/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pellet</t>
-  </si>
-  <si>
-    <t>equipment/mill/pellet/INTERNAL-REVIEW-pellet.html</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>Roll</t>
-  </si>
-  <si>
-    <t>Roll Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/roll/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/roll</t>
-  </si>
-  <si>
-    <t>equipment/mill/roll/INTERNAL-REVIEW-roll.html</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>Shot And Sand</t>
-  </si>
-  <si>
-    <t>Shot and Sand Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/shot-and-sand/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/shot-and-sand</t>
-  </si>
-  <si>
-    <t>equipment/mill/shot-and-sand/INTERNAL-REVIEW-shot-and-sand.html</t>
-  </si>
-  <si>
-    <t>IMS Mill &gt; Shot And Sand (33 listings). IMS also has a separate Mixer-Shot and Sand type, so check the entity overlap.</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>Mixer-Banbury</t>
-  </si>
-  <si>
-    <t>Banbury Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/banbury-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/banbury-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/banbury-mixer/INTERNAL-REVIEW-banbury-mixer.html</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>Mixer-Charge Can and Pony</t>
-  </si>
-  <si>
-    <t>Charge Can and Pony Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/charge-can-and-pony-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/charge-can-and-pony-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/charge-can-and-pony-mixer/INTERNAL-REVIEW-charge-can-and-pony-mixer.html</t>
   </si>
   <si>
     <t>38</t>
@@ -1756,7 +1801,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -1832,7 +1877,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="102" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>39</v>
       </c>
@@ -1908,7 +1953,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>48</v>
       </c>
@@ -1984,7 +2029,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="102" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>57</v>
       </c>
@@ -2062,7 +2107,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>67</v>
       </c>
@@ -2138,7 +2183,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="102" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>75</v>
       </c>
@@ -2216,7 +2261,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>84</v>
       </c>
@@ -2292,7 +2337,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>93</v>
       </c>
@@ -2368,7 +2413,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>102</v>
       </c>
@@ -2444,7 +2489,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>111</v>
       </c>
@@ -2520,7 +2565,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>121</v>
       </c>
@@ -2596,7 +2641,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>130</v>
       </c>
@@ -2672,7 +2717,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>139</v>
       </c>
@@ -2748,7 +2793,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>148</v>
       </c>
@@ -2824,7 +2869,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="19" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>157</v>
       </c>
@@ -2900,7 +2945,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>166</v>
       </c>
@@ -2923,320 +2968,388 @@
       <c r="H20" s="3">
         <v>7</v>
       </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="3"/>
+      <c r="I20" s="3">
+        <v>7</v>
+      </c>
+      <c r="J20" s="3">
+        <v>3</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="L20" s="3">
+        <v>60</v>
+      </c>
       <c r="M20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="R20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="T20" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U20" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V20" s="4"/>
+      <c r="V20" s="5" t="s">
+        <v>172</v>
+      </c>
       <c r="W20" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="X20" s="4"/>
-      <c r="Y20" s="7"/>
-    </row>
-    <row r="21" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>173</v>
+      </c>
+      <c r="X20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y20" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B21" s="3">
         <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="H21" s="3">
         <v>11</v>
       </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="3"/>
+      <c r="I21" s="3">
+        <v>11</v>
+      </c>
+      <c r="J21" s="3">
+        <v>11</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="L21" s="3">
+        <v>600</v>
+      </c>
       <c r="M21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="R21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="S21" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="T21" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U21" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V21" s="4"/>
+      <c r="V21" s="5" t="s">
+        <v>181</v>
+      </c>
       <c r="W21" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="X21" s="4"/>
-      <c r="Y21" s="7"/>
-    </row>
-    <row r="22" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+      <c r="X21" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B22" s="3">
         <v>4</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="H22" s="3">
         <v>24</v>
       </c>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="3"/>
+      <c r="I22" s="3">
+        <v>24</v>
+      </c>
+      <c r="J22" s="3">
+        <v>23</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="L22" s="3">
+        <v>40</v>
+      </c>
       <c r="M22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="R22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="S22" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="T22" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U22" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V22" s="4"/>
+      <c r="V22" s="5" t="s">
+        <v>190</v>
+      </c>
       <c r="W22" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="7"/>
-    </row>
-    <row r="23" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+      <c r="X22" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y22" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B23" s="3">
         <v>4</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="H23" s="3">
         <v>4</v>
       </c>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="3"/>
+      <c r="I23" s="3">
+        <v>4</v>
+      </c>
+      <c r="J23" s="3">
+        <v>3</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="L23" s="3">
+        <v>1100</v>
+      </c>
       <c r="M23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="R23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="T23" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U23" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V23" s="4"/>
+      <c r="V23" s="5" t="s">
+        <v>200</v>
+      </c>
       <c r="W23" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="X23" s="4"/>
+        <v>201</v>
+      </c>
+      <c r="X23" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y23" s="7" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="B24" s="3">
         <v>4</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="H24" s="3">
         <v>12</v>
       </c>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="3"/>
+      <c r="I24" s="3">
+        <v>12</v>
+      </c>
+      <c r="J24" s="3">
+        <v>12</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="L24" s="3">
+        <v>1300</v>
+      </c>
       <c r="M24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="R24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>171</v>
+        <v>33</v>
       </c>
       <c r="T24" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U24" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V24" s="4"/>
+      <c r="V24" s="5" t="s">
+        <v>209</v>
+      </c>
       <c r="W24" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="X24" s="4"/>
-      <c r="Y24" s="7"/>
+        <v>210</v>
+      </c>
+      <c r="X24" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y24" s="7" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="25" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="B25" s="3">
         <v>5</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="H25" s="3">
         <v>5</v>
@@ -3246,25 +3359,25 @@
       <c r="K25" s="4"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3275,34 +3388,34 @@
       </c>
       <c r="V25" s="4"/>
       <c r="W25" s="4" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="X25" s="4"/>
       <c r="Y25" s="7" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="B26" s="3">
         <v>5</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="H26" s="3">
         <v>94</v>
@@ -3312,25 +3425,25 @@
       <c r="K26" s="4"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3341,32 +3454,32 @@
       </c>
       <c r="V26" s="4"/>
       <c r="W26" s="4" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="X26" s="4"/>
       <c r="Y26" s="7"/>
     </row>
-    <row r="27" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B27" s="3">
         <v>0</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="H27" s="3">
         <v>161</v>
@@ -3378,7 +3491,7 @@
         <v>148</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="L27" s="3">
         <v>1100</v>
@@ -3412,39 +3525,39 @@
         <v>34</v>
       </c>
       <c r="V27" s="5" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="W27" s="4" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="X27" s="4" t="s">
         <v>37</v>
       </c>
       <c r="Y27" s="7" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
     </row>
     <row r="28" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="B28" s="3">
         <v>5</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="H28" s="3">
         <v>67</v>
@@ -3454,25 +3567,25 @@
       <c r="K28" s="4"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3483,32 +3596,32 @@
       </c>
       <c r="V28" s="4"/>
       <c r="W28" s="4" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="X28" s="4"/>
       <c r="Y28" s="7"/>
     </row>
     <row r="29" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="B29" s="3">
         <v>5</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="H29" s="3">
         <v>31</v>
@@ -3518,25 +3631,25 @@
       <c r="K29" s="4"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T29" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3547,30 +3660,30 @@
       </c>
       <c r="V29" s="4"/>
       <c r="W29" s="4" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="X29" s="4"/>
       <c r="Y29" s="7"/>
     </row>
     <row r="30" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="B30" s="3">
         <v>5</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="H30" s="3">
         <v>5</v>
@@ -3580,25 +3693,25 @@
       <c r="K30" s="4"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T30" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3609,32 +3722,32 @@
       </c>
       <c r="V30" s="4"/>
       <c r="W30" s="4" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="X30" s="4"/>
       <c r="Y30" s="7" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="B31" s="3">
         <v>6</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="H31" s="3">
         <v>1</v>
@@ -3644,25 +3757,25 @@
       <c r="K31" s="4"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T31" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3673,32 +3786,32 @@
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="4" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="7" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="H32" s="3">
         <v>2</v>
@@ -3708,25 +3821,25 @@
       <c r="K32" s="4"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T32" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3737,32 +3850,32 @@
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="4" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="7" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
     <row r="33" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="B33" s="3">
         <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="H33" s="3">
         <v>2</v>
@@ -3772,25 +3885,25 @@
       <c r="K33" s="4"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3801,34 +3914,34 @@
       </c>
       <c r="V33" s="4"/>
       <c r="W33" s="4" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="X33" s="4"/>
       <c r="Y33" s="7" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="B34" s="3">
         <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="H34" s="3">
         <v>8</v>
@@ -3838,25 +3951,25 @@
       <c r="K34" s="4"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3867,32 +3980,32 @@
       </c>
       <c r="V34" s="4"/>
       <c r="W34" s="4" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="X34" s="4"/>
       <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="B35" s="3">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="H35" s="3">
         <v>14</v>
@@ -3902,25 +4015,25 @@
       <c r="K35" s="4"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T35" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3931,32 +4044,32 @@
       </c>
       <c r="V35" s="4"/>
       <c r="W35" s="4" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
       <c r="X35" s="4"/>
       <c r="Y35" s="7"/>
     </row>
     <row r="36" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
       <c r="B36" s="3">
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
       <c r="H36" s="3">
         <v>1</v>
@@ -3966,25 +4079,25 @@
       <c r="K36" s="4"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3995,34 +4108,34 @@
       </c>
       <c r="V36" s="4"/>
       <c r="W36" s="4" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
       <c r="X36" s="4"/>
       <c r="Y36" s="7" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
     </row>
     <row r="37" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="B37" s="3">
         <v>7</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
@@ -4032,25 +4145,25 @@
       <c r="K37" s="4"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4061,34 +4174,34 @@
       </c>
       <c r="V37" s="4"/>
       <c r="W37" s="4" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="X37" s="4"/>
       <c r="Y37" s="7" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
       <c r="B38" s="3">
         <v>7</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="H38" s="3">
         <v>2</v>
@@ -4098,25 +4211,25 @@
       <c r="K38" s="4"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4127,34 +4240,34 @@
       </c>
       <c r="V38" s="4"/>
       <c r="W38" s="4" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="X38" s="4"/>
       <c r="Y38" s="7" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="B39" s="3">
         <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="H39" s="3">
         <v>6</v>
@@ -4164,25 +4277,25 @@
       <c r="K39" s="4"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4193,32 +4306,32 @@
       </c>
       <c r="V39" s="4"/>
       <c r="W39" s="4" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
       <c r="X39" s="4"/>
       <c r="Y39" s="7"/>
     </row>
     <row r="40" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="B40" s="3">
         <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="H40" s="3">
         <v>33</v>
@@ -4228,25 +4341,25 @@
       <c r="K40" s="4"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T40" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4257,32 +4370,32 @@
       </c>
       <c r="V40" s="4"/>
       <c r="W40" s="4" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
       <c r="X40" s="4"/>
       <c r="Y40" s="7" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
     </row>
     <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
       <c r="B41" s="3">
         <v>8</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>306</v>
+        <v>320</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="H41" s="3">
         <v>9</v>
@@ -4292,25 +4405,25 @@
       <c r="K41" s="4"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4321,30 +4434,30 @@
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="X41" s="4"/>
       <c r="Y41" s="7"/>
     </row>
     <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
@@ -4354,25 +4467,25 @@
       <c r="K42" s="4"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4383,32 +4496,32 @@
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="X42" s="4"/>
       <c r="Y42" s="7" t="s">
-        <v>192</v>
+        <v>331</v>
       </c>
     </row>
     <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
@@ -4418,25 +4531,25 @@
       <c r="K43" s="4"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4447,32 +4560,32 @@
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="X43" s="4"/>
       <c r="Y43" s="7" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
@@ -4482,25 +4595,25 @@
       <c r="K44" s="4"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4511,11 +4624,11 @@
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="X44" s="4"/>
       <c r="Y44" s="7" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -4610,55 +4723,60 @@
     <hyperlink ref="V19" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
     <hyperlink ref="F20" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
     <hyperlink ref="G20" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="F21" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="G21" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="F22" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="G22" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="F23" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="G23" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="F24" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="G24" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="F25" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="G25" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="F26" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="G26" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="F27" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="G27" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="V27" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="F28" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="G28" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="F29" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="G29" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="F30" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="G30" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="F31" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="G31" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="F32" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="G32" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="F33" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="G33" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="F34" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="G34" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="F35" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="G35" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="F36" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="G36" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="F37" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="G37" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="F38" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="G38" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="F39" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="G39" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="F40" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="G40" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="F41" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="G41" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="F42" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="G42" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="F43" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="G43" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="F44" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="G44" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="V20" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="F21" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="G21" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="V21" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="F22" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="G22" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="V22" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="F23" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="G23" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="V23" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="F24" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="G24" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="V24" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="F25" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="G25" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="F26" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="G26" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="F27" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="G27" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="V27" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="F28" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="G28" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="F29" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="G29" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="F30" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="G30" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="F31" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="G31" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="F32" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="G32" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="F33" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="G33" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="F34" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="G34" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="F35" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="G35" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="F36" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="G36" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="F37" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="G37" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="F38" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="G38" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="F39" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="G39" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="F40" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="G40" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="F41" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="G41" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="F42" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="G42" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="F43" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="G43" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="F44" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="G44" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4678,25 +4796,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -4705,16 +4823,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -4723,16 +4841,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -4741,7 +4859,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -4750,7 +4868,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -4759,27 +4877,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>395</v>
+        <v>453</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4788,11 +4906,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -4801,11 +4919,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -4814,11 +4932,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4827,11 +4945,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -4840,11 +4958,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -4853,11 +4971,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -4866,16 +4984,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -4883,16 +5001,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -4989,7 +5107,7 @@
       </c>
       <c r="C30" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A30,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D30" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A30,Pages!$U$5:$U$44,"Approved")</f>
@@ -4997,7 +5115,7 @@
       </c>
       <c r="E30" s="6" t="str">
         <f>IF(D30=B30,"Approved",IF(C30=B30,"Ready for client review",IF(C30&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A30,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -5100,15 +5218,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5116,7 +5234,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -5124,7 +5242,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -5132,7 +5250,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5140,7 +5258,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -5148,7 +5266,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5156,7 +5274,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -5164,7 +5282,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5172,28 +5290,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Tracker: batch 5 (P20-25) ready for client review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A55A780-B555-4C03-AF81-02F95ADEDFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD1C5C4E-FA59-4D97-967E-9EB0024965C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="393">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -694,127 +694,169 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/air-fin</t>
   </si>
   <si>
+    <t>air cooled heat exchanger</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/air-fin/</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/air-fin/INTERNAL-REVIEW-air-fin.html</t>
+  </si>
+  <si>
+    <t>Built as 'Air Cooled Heat Exchangers' from 5 units: Balke Durr fin fan coolers of 2,100 m2, Hiross Hypercool units and a Finnco ambient air vaporizer. Duty and gas-service notes stay off the page. Comparison links the live shell and tube page. Cleaning, fouling and maintenance terms are excluded (client rule).</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>Block</t>
+  </si>
+  <si>
+    <t>Block Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/block/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/block</t>
+  </si>
+  <si>
+    <t>graphite heat exchanger</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/block/</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/block/INTERNAL-REVIEW-block.html</t>
+  </si>
+  <si>
+    <t>Built as 'Graphite Block Heat Exchangers' from 94 listings: Ralph Coidan, Carbone Lorraine, Vicarb, GAB Neumann, SGL Carbon and others, plus Karbate tube units and an unused Chart BAHX. One listing's test note stays off (no-defects rule). IMS files Vicarb, Carbone and GAB units under several maker records, so those tabs link IMS keyword searches. Manufacturer domains (SGL) were kept out of the competitor set so the brand blocklist does not block them.</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Plate and Frame</t>
+  </si>
+  <si>
+    <t>Plate and Frame Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/plate-and-frame/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/plate-and-frame</t>
+  </si>
+  <si>
+    <t>plate and frame heat exchanger</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/plate-and-frame/</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/plate-and-frame/INTERNAL-REVIEW-plate-and-frame.html</t>
+  </si>
+  <si>
+    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Spiral</t>
+  </si>
+  <si>
+    <t>Spiral Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/spiral/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/spiral</t>
+  </si>
+  <si>
+    <t>spiral heat exchanger</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/spiral/</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/spiral/INTERNAL-REVIEW-spiral.html</t>
+  </si>
+  <si>
+    <t>Built from 67 listings: Alfa Laval spiral plate units (to 205.8 m2), Kuhni coil exchangers, QVF and Schott glass, GAB Neumann graphite, GEA Canzler, American Heat Reclaiming and others. Comparison: spiral plate vs spiral tube (both in stock). Alfa Laval and American Heat Reclaiming tabs link keyword searches (spelling variants on IMS).</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>Welded Plate</t>
+  </si>
+  <si>
+    <t>Welded Plate Heat Exchangers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/welded-plate/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/welded-plate</t>
+  </si>
+  <si>
+    <t>welded plate heat exchanger</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/welded-plate/</t>
+  </si>
+  <si>
+    <t>equipment/heat-exchanger/welded-plate/INTERNAL-REVIEW-welded-plate.html</t>
+  </si>
+  <si>
+    <t>Built from 31 listings: Alfa Laval Compabloc CP30, CPL30, CPL20, CPF, CPK40 and unused CPX50 and CPX75 units, plus Kapp. The CPX50 plate grade is not published (IMS fields disagree). Comparison links the plate and frame pilot page (new URL, publish together). Semi-welded terms are excluded (no units).</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Homogenizer</t>
+  </si>
+  <si>
+    <t>Homogenizers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/homogenizer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/homogenizer</t>
+  </si>
+  <si>
+    <t>industrial homogenizer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/homogenizer/</t>
+  </si>
+  <si>
+    <t>equipment/homogenizer/INTERNAL-REVIEW-homogenizer.html</t>
+  </si>
+  <si>
+    <t>Built as 'Industrial Homogenizers' from 5 units: SPX, Rannie and APV Gaulin high-pressure machines and BWS and Hoelschertechnik rotor-stator units, split by type tabs on IMS pressure filters. Lab-instrument and application terms are excluded; 'homogenizer' (1,500) is a lab-heavy head term.</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Incinerator</t>
+  </si>
+  <si>
+    <t>Incinerators</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/incinerator/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/incinerator</t>
+  </si>
+  <si>
     <t>Not started</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/air-fin/INTERNAL-REVIEW-air-fin.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 5 units.</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>Block</t>
-  </si>
-  <si>
-    <t>Block Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/block/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/block</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/block/INTERNAL-REVIEW-block.html</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>Plate and Frame</t>
-  </si>
-  <si>
-    <t>Plate and Frame Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/plate-and-frame/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/plate-and-frame</t>
-  </si>
-  <si>
-    <t>plate and frame heat exchanger</t>
-  </si>
-  <si>
-    <t>https://international-process-plants-update-one.vercel.app/equipment/heat-exchanger/plate-and-frame/</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/plate-and-frame/INTERNAL-REVIEW-plate-and-frame.html</t>
-  </si>
-  <si>
-    <t>Pilot. Rev 4 approved internally on 2026-10-01 (rev 1 copy, live reactor layout, IMS listing). It is the model for the other 39 pages. 2026-10-02: live hero, logo strip and tabs; blog and intro links removed; hero predicates varied. Hero opener rewritten on 2026-10-02 to the client's 'Buying ... from IPP [verb] ... while [verb]ing issues like ...' format; review doc re-issued. Live white header with the IPP logo and menu added on 2026-10-02 (adbac2f).</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>Spiral</t>
-  </si>
-  <si>
-    <t>Spiral Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/spiral/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/spiral</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/spiral/INTERNAL-REVIEW-spiral.html</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>Welded Plate</t>
-  </si>
-  <si>
-    <t>Welded Plate Heat Exchangers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/heat-exchanger/welded-plate/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/heat-exchanger/welded-plate</t>
-  </si>
-  <si>
-    <t>equipment/heat-exchanger/welded-plate/INTERNAL-REVIEW-welded-plate.html</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>Homogenizer</t>
-  </si>
-  <si>
-    <t>Homogenizers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/homogenizer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/homogenizer</t>
-  </si>
-  <si>
-    <t>equipment/homogenizer/INTERNAL-REVIEW-homogenizer.html</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>Incinerator</t>
-  </si>
-  <si>
-    <t>Incinerators</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/incinerator/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/incinerator</t>
   </si>
   <si>
     <t>equipment/incinerator/INTERNAL-REVIEW-incinerator.html</t>
@@ -3329,7 +3371,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>212</v>
       </c>
@@ -3354,50 +3396,62 @@
       <c r="H25" s="3">
         <v>5</v>
       </c>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="3"/>
+      <c r="I25" s="3">
+        <v>5</v>
+      </c>
+      <c r="J25" s="3">
+        <v>4</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="L25" s="3">
+        <v>300</v>
+      </c>
       <c r="M25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="R25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="T25" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U25" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V25" s="4"/>
+      <c r="V25" s="5" t="s">
+        <v>219</v>
+      </c>
       <c r="W25" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="X25" s="4"/>
+        <v>220</v>
+      </c>
+      <c r="X25" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y25" s="7" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="26" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B26" s="3">
         <v>5</v>
@@ -3406,62 +3460,76 @@
         <v>213</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H26" s="3">
         <v>94</v>
       </c>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="3"/>
+      <c r="I26" s="3">
+        <v>94</v>
+      </c>
+      <c r="J26" s="3">
+        <v>91</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="L26" s="3">
+        <v>200</v>
+      </c>
       <c r="M26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="R26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="T26" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U26" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V26" s="4"/>
+      <c r="V26" s="5" t="s">
+        <v>228</v>
+      </c>
       <c r="W26" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="X26" s="4"/>
-      <c r="Y26" s="7"/>
+        <v>229</v>
+      </c>
+      <c r="X26" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y26" s="7" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="27" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B27" s="3">
         <v>0</v>
@@ -3470,16 +3538,16 @@
         <v>213</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="H27" s="3">
         <v>161</v>
@@ -3491,7 +3559,7 @@
         <v>148</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="L27" s="3">
         <v>1100</v>
@@ -3525,21 +3593,21 @@
         <v>34</v>
       </c>
       <c r="V27" s="5" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="W27" s="4" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="X27" s="4" t="s">
         <v>37</v>
       </c>
       <c r="Y27" s="7" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="28" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B28" s="3">
         <v>5</v>
@@ -3548,62 +3616,76 @@
         <v>213</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="H28" s="3">
         <v>67</v>
       </c>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="3"/>
+      <c r="I28" s="3">
+        <v>67</v>
+      </c>
+      <c r="J28" s="3">
+        <v>63</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="L28" s="3">
+        <v>350</v>
+      </c>
       <c r="M28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="R28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="T28" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U28" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V28" s="4"/>
+      <c r="V28" s="5" t="s">
+        <v>246</v>
+      </c>
       <c r="W28" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="X28" s="4"/>
-      <c r="Y28" s="7"/>
-    </row>
-    <row r="29" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>247</v>
+      </c>
+      <c r="X28" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y28" s="7" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B29" s="3">
         <v>5</v>
@@ -3612,142 +3694,168 @@
         <v>213</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="H29" s="3">
         <v>31</v>
       </c>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="3"/>
+      <c r="I29" s="3">
+        <v>31</v>
+      </c>
+      <c r="J29" s="3">
+        <v>30</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="L29" s="3">
+        <v>150</v>
+      </c>
       <c r="M29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="R29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="T29" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U29" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V29" s="4"/>
+      <c r="V29" s="5" t="s">
+        <v>255</v>
+      </c>
       <c r="W29" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="X29" s="4"/>
-      <c r="Y29" s="7"/>
-    </row>
-    <row r="30" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>256</v>
+      </c>
+      <c r="X29" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y29" s="7" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="B30" s="3">
         <v>5</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="H30" s="3">
         <v>5</v>
       </c>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="3"/>
+      <c r="I30" s="3">
+        <v>5</v>
+      </c>
+      <c r="J30" s="3">
+        <v>5</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="L30" s="3">
+        <v>150</v>
+      </c>
       <c r="M30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="R30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>218</v>
+        <v>33</v>
       </c>
       <c r="T30" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U30" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V30" s="4"/>
+      <c r="V30" s="5" t="s">
+        <v>264</v>
+      </c>
       <c r="W30" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="X30" s="4"/>
+        <v>265</v>
+      </c>
+      <c r="X30" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y30" s="7" t="s">
-        <v>220</v>
+        <v>266</v>
       </c>
     </row>
     <row r="31" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="B31" s="3">
         <v>6</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="H31" s="3">
         <v>1</v>
@@ -3757,25 +3865,25 @@
       <c r="K31" s="4"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T31" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3786,32 +3894,32 @@
       </c>
       <c r="V31" s="4"/>
       <c r="W31" s="4" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="X31" s="4"/>
       <c r="Y31" s="7" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="H32" s="3">
         <v>2</v>
@@ -3821,25 +3929,25 @@
       <c r="K32" s="4"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T32" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3850,32 +3958,32 @@
       </c>
       <c r="V32" s="4"/>
       <c r="W32" s="4" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="X32" s="4"/>
       <c r="Y32" s="7" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
     </row>
     <row r="33" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="B33" s="3">
         <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
       <c r="H33" s="3">
         <v>2</v>
@@ -3885,25 +3993,25 @@
       <c r="K33" s="4"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3914,34 +4022,34 @@
       </c>
       <c r="V33" s="4"/>
       <c r="W33" s="4" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
       <c r="X33" s="4"/>
       <c r="Y33" s="7" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
     </row>
     <row r="34" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B34" s="3">
         <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="H34" s="3">
         <v>8</v>
@@ -3951,25 +4059,25 @@
       <c r="K34" s="4"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3980,32 +4088,32 @@
       </c>
       <c r="V34" s="4"/>
       <c r="W34" s="4" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
       <c r="X34" s="4"/>
       <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="B35" s="3">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
       <c r="H35" s="3">
         <v>14</v>
@@ -4015,25 +4123,25 @@
       <c r="K35" s="4"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T35" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4044,32 +4152,32 @@
       </c>
       <c r="V35" s="4"/>
       <c r="W35" s="4" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
       <c r="X35" s="4"/>
       <c r="Y35" s="7"/>
     </row>
     <row r="36" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="B36" s="3">
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="H36" s="3">
         <v>1</v>
@@ -4079,25 +4187,25 @@
       <c r="K36" s="4"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4108,34 +4216,34 @@
       </c>
       <c r="V36" s="4"/>
       <c r="W36" s="4" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="X36" s="4"/>
       <c r="Y36" s="7" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
     </row>
     <row r="37" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
       <c r="B37" s="3">
         <v>7</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
@@ -4145,25 +4253,25 @@
       <c r="K37" s="4"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4174,34 +4282,34 @@
       </c>
       <c r="V37" s="4"/>
       <c r="W37" s="4" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="X37" s="4"/>
       <c r="Y37" s="7" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
       <c r="B38" s="3">
         <v>7</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="H38" s="3">
         <v>2</v>
@@ -4211,25 +4319,25 @@
       <c r="K38" s="4"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4240,34 +4348,34 @@
       </c>
       <c r="V38" s="4"/>
       <c r="W38" s="4" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
       <c r="X38" s="4"/>
       <c r="Y38" s="7" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>306</v>
+        <v>320</v>
       </c>
       <c r="B39" s="3">
         <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="H39" s="3">
         <v>6</v>
@@ -4277,25 +4385,25 @@
       <c r="K39" s="4"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4306,32 +4414,32 @@
       </c>
       <c r="V39" s="4"/>
       <c r="W39" s="4" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="X39" s="4"/>
       <c r="Y39" s="7"/>
     </row>
     <row r="40" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="B40" s="3">
         <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="H40" s="3">
         <v>33</v>
@@ -4341,25 +4449,25 @@
       <c r="K40" s="4"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T40" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4370,32 +4478,32 @@
       </c>
       <c r="V40" s="4"/>
       <c r="W40" s="4" t="s">
-        <v>317</v>
+        <v>331</v>
       </c>
       <c r="X40" s="4"/>
       <c r="Y40" s="7" t="s">
-        <v>318</v>
+        <v>332</v>
       </c>
     </row>
     <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="B41" s="3">
         <v>8</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>320</v>
+        <v>334</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>322</v>
+        <v>336</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="H41" s="3">
         <v>9</v>
@@ -4405,25 +4513,25 @@
       <c r="K41" s="4"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4434,30 +4542,30 @@
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="X41" s="4"/>
       <c r="Y41" s="7"/>
     </row>
     <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>325</v>
+        <v>339</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>326</v>
+        <v>340</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>327</v>
+        <v>341</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>328</v>
+        <v>342</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>329</v>
+        <v>343</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
@@ -4467,25 +4575,25 @@
       <c r="K42" s="4"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4496,32 +4604,32 @@
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4" t="s">
-        <v>330</v>
+        <v>344</v>
       </c>
       <c r="X42" s="4"/>
       <c r="Y42" s="7" t="s">
-        <v>331</v>
+        <v>345</v>
       </c>
     </row>
     <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>332</v>
+        <v>346</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>333</v>
+        <v>347</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>334</v>
+        <v>348</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>335</v>
+        <v>349</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
@@ -4531,25 +4639,25 @@
       <c r="K43" s="4"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4560,32 +4668,32 @@
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4" t="s">
-        <v>337</v>
+        <v>351</v>
       </c>
       <c r="X43" s="4"/>
       <c r="Y43" s="7" t="s">
-        <v>338</v>
+        <v>352</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>339</v>
+        <v>353</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>340</v>
+        <v>354</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>342</v>
+        <v>356</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
@@ -4595,25 +4703,25 @@
       <c r="K44" s="4"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4624,11 +4732,11 @@
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4" t="s">
-        <v>344</v>
+        <v>358</v>
       </c>
       <c r="X44" s="4"/>
       <c r="Y44" s="7" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -4738,45 +4846,50 @@
     <hyperlink ref="V24" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
     <hyperlink ref="F25" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
     <hyperlink ref="G25" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="F26" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="G26" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="F27" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="G27" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="V27" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="F28" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="G28" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="F29" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="G29" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="F30" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="G30" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="F31" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="G31" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="F32" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="G32" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="F33" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="G33" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="F34" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="G34" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="F35" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="G35" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="F36" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="G36" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="F37" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="G37" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="F38" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="G38" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="F39" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="G39" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="F40" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="G40" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="F41" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="G41" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="F42" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="G42" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="F43" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="G43" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="F44" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="G44" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="V25" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="F26" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="G26" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="V26" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="F27" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="G27" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="V27" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="F28" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="G28" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="V28" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="F29" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="G29" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="V29" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="F30" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="G30" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="V30" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="F31" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="G31" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="F32" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="G32" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="F33" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="G33" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="F34" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="G34" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="F35" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="G35" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="F36" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="G36" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="F37" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="G37" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="F38" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="G38" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="F39" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="G39" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="F40" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="G40" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="F41" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="G41" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="F42" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="G42" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="F43" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="G43" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="F44" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="G44" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4796,25 +4909,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>345</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>346</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>347</v>
+        <v>361</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>348</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>349</v>
+        <v>363</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -4823,16 +4936,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>350</v>
+        <v>364</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>351</v>
+        <v>365</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -4841,16 +4954,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>218</v>
+        <v>272</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>352</v>
+        <v>366</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -4859,7 +4972,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>353</v>
+        <v>367</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -4868,7 +4981,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -4877,27 +4990,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>453</v>
+        <v>655</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>358</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4906,11 +5019,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -4919,11 +5032,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -4932,11 +5045,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4945,11 +5058,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -4958,11 +5071,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -4971,11 +5084,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -4984,16 +5097,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.52500000000000002</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>359</v>
+        <v>373</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5001,16 +5114,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>360</v>
+        <v>374</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>350</v>
+        <v>364</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>361</v>
+        <v>375</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>362</v>
+        <v>376</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -5128,7 +5241,7 @@
       </c>
       <c r="C31" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A31,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D31" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A31,Pages!$U$5:$U$44,"Approved")</f>
@@ -5136,7 +5249,7 @@
       </c>
       <c r="E31" s="6" t="str">
         <f>IF(D31=B31,"Approved",IF(C31=B31,"Ready for client review",IF(C31&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A31,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -5218,15 +5331,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>363</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>365</v>
+        <v>379</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5234,7 +5347,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>366</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -5242,7 +5355,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>367</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -5250,7 +5363,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>368</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5258,7 +5371,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>369</v>
+        <v>383</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -5266,7 +5379,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>370</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5274,7 +5387,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>371</v>
+        <v>385</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -5282,7 +5395,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>372</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5290,28 +5403,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>374</v>
+        <v>388</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>375</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>376</v>
+        <v>390</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>377</v>
+        <v>391</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>378</v>
+        <v>392</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Tracker: batch 6 (P26-30) ready for client review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD1C5C4E-FA59-4D97-967E-9EB0024965C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08A65D6-253B-431C-AE00-5B33E459B806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="408">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -856,148 +856,193 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/incinerator</t>
   </si>
   <si>
+    <t>thermal oxidizer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/incinerator/</t>
+  </si>
+  <si>
+    <t>equipment/incinerator/INTERNAL-REVIEW-incinerator.html</t>
+  </si>
+  <si>
+    <t>Built as 'Incinerators &amp; Thermal Oxidizers' around one good used Thermatrix ES-100 flameless thermal oxidizer, so the page leans on sourcing to specification. 'thermal oxidizer' (900) leads; animal, pet and cremation incinerator demand is excluded. Comparison: flameless vs direct-fired. IMS's ES-100 dimensions (47.2 m high) and 'Liquid' phase field are not credible and stay off the page.</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>Kettle</t>
+  </si>
+  <si>
+    <t>Kettles</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/kettle/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kettle</t>
+  </si>
+  <si>
+    <t>steam jacketed kettle</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/kettle/</t>
+  </si>
+  <si>
+    <t>equipment/kettle/INTERNAL-REVIEW-kettle.html</t>
+  </si>
+  <si>
+    <t>Built as 'Steam Jacketed Kettles' from two good used Groen units (TA25SP mixer kettle, TDC/2-20 table-top kettle). Foodservice brands not in stock (Cleveland, Vulcan, Market Forge) are excluded. Comparison vs jacketed reactors links the live reactor hub. IMS's TDC jacket (carbon steel) and bottom-head (stainless steel 904) fields conflict with its 304 build, so only the overall material is published.</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Kiln</t>
+  </si>
+  <si>
+    <t>Kilns</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/kiln/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kiln</t>
+  </si>
+  <si>
+    <t>rotary kiln</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/kiln/</t>
+  </si>
+  <si>
+    <t>equipment/kiln/INTERNAL-REVIEW-kiln.html</t>
+  </si>
+  <si>
+    <t>Built as 'Rotary Kilns' from two good used units: a Bethlehem indirect-fired Inconel kiln and a nickel kiln with no maker named. 'rotary kiln' (2,100) leads; cement, lime, incineration and refractory demand is excluded. Comparison: indirect vs direct-fired. Firing type is stated only for the Bethlehem unit.</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>Mill</t>
+  </si>
+  <si>
+    <t>Ball</t>
+  </si>
+  <si>
+    <t>Ball Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/ball/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/ball</t>
+  </si>
+  <si>
+    <t>ball mill</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/ball/</t>
+  </si>
+  <si>
+    <t>equipment/mill/ball/INTERNAL-REVIEW-ball.html</t>
+  </si>
+  <si>
+    <t>Built from good used Blaw Knox Ni-hard lined cylindrical mills, Hardinge conical mills, a TEMA vibratory mill, a rod mill and an Engineering Plastics pilot mill, with manufacturer tabs for Blaw Knox and Hardinge. Comparison: conical vs cylindrical. IMS's 25.4 mm rod-mill diameter and the Hardinge 'approximately 470 mm' ends stay off the page; no throughput claims.</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Colloid</t>
+  </si>
+  <si>
+    <t>Colloid Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/colloid/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/colloid</t>
+  </si>
+  <si>
+    <t>colloid mill</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/colloid/</t>
+  </si>
+  <si>
+    <t>equipment/mill/colloid/INTERNAL-REVIEW-colloid.html</t>
+  </si>
+  <si>
+    <t>Built from IMS's mixed colloid category: rotor-stator colloid and dispersion mills (IKA-Werk, Premier), Peters &amp; Smith attritors and Alpine, Williams, Reitz and Bepex hammer mills, split by type tabs, plus a new GPS Multi-Mill. No condition tabs. Comparison vs high-pressure homogenizers links the new homogenizer page.</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Kady</t>
+  </si>
+  <si>
+    <t>Kady Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/kady/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/kady</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>equipment/incinerator/INTERNAL-REVIEW-incinerator.html</t>
+    <t>equipment/mill/kady/INTERNAL-REVIEW-kady.html</t>
   </si>
   <si>
     <t>Thin inventory: 1 unit on IMS.</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>Kettle</t>
-  </si>
-  <si>
-    <t>Kettles</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/kettle/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kettle</t>
-  </si>
-  <si>
-    <t>equipment/kettle/INTERNAL-REVIEW-kettle.html</t>
+    <t>32</t>
+  </si>
+  <si>
+    <t>Pebble</t>
+  </si>
+  <si>
+    <t>Pebble Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/pebble/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pebble</t>
+  </si>
+  <si>
+    <t>equipment/mill/pebble/INTERNAL-REVIEW-pebble.html</t>
+  </si>
+  <si>
+    <t>IMS shows 0 units. The page will be a sourcing page with no listing.</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Pellet</t>
+  </si>
+  <si>
+    <t>Pellet Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/pellet/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pellet</t>
+  </si>
+  <si>
+    <t>equipment/mill/pellet/INTERNAL-REVIEW-pellet.html</t>
   </si>
   <si>
     <t>Thin inventory: 2 units.</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>Kiln</t>
-  </si>
-  <si>
-    <t>Kilns</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/kiln/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/kiln</t>
-  </si>
-  <si>
-    <t>equipment/kiln/INTERNAL-REVIEW-kiln.html</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>Mill</t>
-  </si>
-  <si>
-    <t>Ball</t>
-  </si>
-  <si>
-    <t>Ball Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/ball/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/ball</t>
-  </si>
-  <si>
-    <t>equipment/mill/ball/INTERNAL-REVIEW-ball.html</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Colloid</t>
-  </si>
-  <si>
-    <t>Colloid Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/colloid/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/colloid</t>
-  </si>
-  <si>
-    <t>equipment/mill/colloid/INTERNAL-REVIEW-colloid.html</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>Kady</t>
-  </si>
-  <si>
-    <t>Kady Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/kady/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/kady</t>
-  </si>
-  <si>
-    <t>equipment/mill/kady/INTERNAL-REVIEW-kady.html</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>Pebble</t>
-  </si>
-  <si>
-    <t>Pebble Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/pebble/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pebble</t>
-  </si>
-  <si>
-    <t>equipment/mill/pebble/INTERNAL-REVIEW-pebble.html</t>
-  </si>
-  <si>
-    <t>IMS shows 0 units. The page will be a sourcing page with no listing.</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>Pellet</t>
-  </si>
-  <si>
-    <t>Pellet Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/pellet/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pellet</t>
-  </si>
-  <si>
-    <t>equipment/mill/pellet/INTERNAL-REVIEW-pellet.html</t>
   </si>
   <si>
     <t>34</t>
@@ -3837,7 +3882,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="31" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>267</v>
       </c>
@@ -3860,324 +3905,388 @@
       <c r="H31" s="3">
         <v>1</v>
       </c>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="3"/>
+      <c r="I31" s="3">
+        <v>1</v>
+      </c>
+      <c r="J31" s="3">
+        <v>1</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="L31" s="3">
+        <v>900</v>
+      </c>
       <c r="M31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="N31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="T31" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U31" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V31" s="4"/>
+      <c r="V31" s="5" t="s">
+        <v>273</v>
+      </c>
       <c r="W31" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="X31" s="4"/>
+        <v>274</v>
+      </c>
+      <c r="X31" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y31" s="7" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="32" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H32" s="3">
         <v>2</v>
       </c>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="3"/>
+      <c r="I32" s="3">
+        <v>2</v>
+      </c>
+      <c r="J32" s="3">
+        <v>2</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="L32" s="3">
+        <v>1000</v>
+      </c>
       <c r="M32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="R32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="T32" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U32" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V32" s="4"/>
+      <c r="V32" s="5" t="s">
+        <v>282</v>
+      </c>
       <c r="W32" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="X32" s="4"/>
+        <v>283</v>
+      </c>
+      <c r="X32" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y32" s="7" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="33" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B33" s="3">
         <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="H33" s="3">
         <v>2</v>
       </c>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="3"/>
+      <c r="I33" s="3">
+        <v>2</v>
+      </c>
+      <c r="J33" s="3">
+        <v>2</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="L33" s="3">
+        <v>2100</v>
+      </c>
       <c r="M33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="P33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="Q33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="R33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="T33" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U33" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V33" s="4"/>
+      <c r="V33" s="5" t="s">
+        <v>291</v>
+      </c>
       <c r="W33" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="X33" s="4"/>
+        <v>292</v>
+      </c>
+      <c r="X33" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y33" s="7" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="34" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="B34" s="3">
         <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="H34" s="3">
         <v>8</v>
       </c>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="3"/>
+      <c r="I34" s="3">
+        <v>8</v>
+      </c>
+      <c r="J34" s="3">
+        <v>8</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="L34" s="3">
+        <v>1600</v>
+      </c>
       <c r="M34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="N34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="R34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="T34" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U34" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V34" s="4"/>
+      <c r="V34" s="5" t="s">
+        <v>301</v>
+      </c>
       <c r="W34" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="X34" s="4"/>
-      <c r="Y34" s="7"/>
-    </row>
-    <row r="35" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>302</v>
+      </c>
+      <c r="X34" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y34" s="7" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="B35" s="3">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="H35" s="3">
         <v>14</v>
       </c>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="3"/>
+      <c r="I35" s="3">
+        <v>14</v>
+      </c>
+      <c r="J35" s="3">
+        <v>12</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="L35" s="3">
+        <v>300</v>
+      </c>
       <c r="M35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="R35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>272</v>
+        <v>33</v>
       </c>
       <c r="T35" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U35" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V35" s="4"/>
+      <c r="V35" s="5" t="s">
+        <v>310</v>
+      </c>
       <c r="W35" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="X35" s="4"/>
-      <c r="Y35" s="7"/>
+        <v>311</v>
+      </c>
+      <c r="X35" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>312</v>
+      </c>
     </row>
     <row r="36" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="B36" s="3">
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="H36" s="3">
         <v>1</v>
@@ -4187,25 +4296,25 @@
       <c r="K36" s="4"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4216,34 +4325,34 @@
       </c>
       <c r="V36" s="4"/>
       <c r="W36" s="4" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="X36" s="4"/>
       <c r="Y36" s="7" t="s">
-        <v>274</v>
+        <v>320</v>
       </c>
     </row>
     <row r="37" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="B37" s="3">
         <v>7</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
@@ -4253,25 +4362,25 @@
       <c r="K37" s="4"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4282,34 +4391,34 @@
       </c>
       <c r="V37" s="4"/>
       <c r="W37" s="4" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="X37" s="4"/>
       <c r="Y37" s="7" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="B38" s="3">
         <v>7</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>317</v>
+        <v>331</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>318</v>
+        <v>332</v>
       </c>
       <c r="H38" s="3">
         <v>2</v>
@@ -4319,25 +4428,25 @@
       <c r="K38" s="4"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4348,34 +4457,34 @@
       </c>
       <c r="V38" s="4"/>
       <c r="W38" s="4" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="X38" s="4"/>
       <c r="Y38" s="7" t="s">
-        <v>281</v>
+        <v>334</v>
       </c>
     </row>
     <row r="39" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="B39" s="3">
         <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="H39" s="3">
         <v>6</v>
@@ -4385,25 +4494,25 @@
       <c r="K39" s="4"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4414,32 +4523,32 @@
       </c>
       <c r="V39" s="4"/>
       <c r="W39" s="4" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="X39" s="4"/>
       <c r="Y39" s="7"/>
     </row>
     <row r="40" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="B40" s="3">
         <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="H40" s="3">
         <v>33</v>
@@ -4449,25 +4558,25 @@
       <c r="K40" s="4"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T40" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4478,32 +4587,32 @@
       </c>
       <c r="V40" s="4"/>
       <c r="W40" s="4" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="X40" s="4"/>
       <c r="Y40" s="7" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
     </row>
     <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="B41" s="3">
         <v>8</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="H41" s="3">
         <v>9</v>
@@ -4513,25 +4622,25 @@
       <c r="K41" s="4"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4542,30 +4651,30 @@
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="X41" s="4"/>
       <c r="Y41" s="7"/>
     </row>
     <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
@@ -4575,25 +4684,25 @@
       <c r="K42" s="4"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4604,32 +4713,32 @@
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="X42" s="4"/>
       <c r="Y42" s="7" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
@@ -4639,25 +4748,25 @@
       <c r="K43" s="4"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4668,32 +4777,32 @@
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="X43" s="4"/>
       <c r="Y43" s="7" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
@@ -4703,25 +4812,25 @@
       <c r="K44" s="4"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4732,11 +4841,11 @@
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="X44" s="4"/>
       <c r="Y44" s="7" t="s">
-        <v>281</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -4864,32 +4973,37 @@
     <hyperlink ref="V30" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
     <hyperlink ref="F31" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
     <hyperlink ref="G31" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="F32" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="G32" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="F33" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="G33" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="F34" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="G34" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="F35" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="G35" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="F36" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="G36" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="F37" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="G37" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="F38" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="G38" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="F39" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="G39" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="F40" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="G40" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="F41" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="G41" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="F42" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
-    <hyperlink ref="G42" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
-    <hyperlink ref="F43" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
-    <hyperlink ref="G43" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
-    <hyperlink ref="F44" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
-    <hyperlink ref="G44" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="V31" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="F32" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="G32" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="V32" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="F33" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="G33" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="V33" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="F34" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="G34" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="V34" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="F35" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="G35" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="V35" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="F36" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="G36" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="F37" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="G37" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="F38" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="G38" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="F39" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="G39" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="F40" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="G40" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="F41" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="G41" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="F42" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="G42" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="F43" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="G43" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="F44" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="G44" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4909,25 +5023,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -4936,16 +5050,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -4954,16 +5068,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>272</v>
+        <v>318</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -4972,7 +5086,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -4981,7 +5095,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -4990,27 +5104,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>655</v>
+        <v>682</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -5019,11 +5133,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -5032,11 +5146,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5045,11 +5159,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -5058,11 +5172,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -5071,11 +5185,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -5084,11 +5198,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -5097,16 +5211,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.65</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5114,16 +5228,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -5262,7 +5376,7 @@
       </c>
       <c r="C32" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A32,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D32" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A32,Pages!$U$5:$U$44,"Approved")</f>
@@ -5270,7 +5384,7 @@
       </c>
       <c r="E32" s="6" t="str">
         <f>IF(D32=B32,"Approved",IF(C32=B32,"Ready for client review",IF(C32&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A32,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -5331,15 +5445,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5347,7 +5461,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -5355,7 +5469,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -5363,7 +5477,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5371,7 +5485,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -5379,7 +5493,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5387,7 +5501,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -5395,7 +5509,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5403,28 +5517,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Tracker: batch 7 (P31-35) ready for client review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08A65D6-253B-431C-AE00-5B33E459B806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4D0BB7-A446-4F86-AA3A-64ADA71C3B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="420">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -994,172 +994,208 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/kady</t>
   </si>
   <si>
+    <t>kady mill</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/kady/</t>
+  </si>
+  <si>
+    <t>equipment/mill/kady/INTERNAL-REVIEW-kady.html</t>
+  </si>
+  <si>
+    <t>IMS's Kady category holds no Kady dispersion mill: its listing is a Powtec RTS 350 x 300 rotor sieving mill, so the page is built as 'Kady &amp; Rotor Sieve Mills', names the Powtec for what it is and offers Kady mills through sourcing to specification. 'kady mill' (50) is the only measurable machine term ('kady' alone is people's names). The listing's ATEX/Ex wording, motor marking and throughput figure stay off the page.</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>Pebble</t>
+  </si>
+  <si>
+    <t>Pebble Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/pebble/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pebble</t>
+  </si>
+  <si>
+    <t>pebble mills</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/pebble/</t>
+  </si>
+  <si>
+    <t>equipment/mill/pebble/INTERNAL-REVIEW-pebble.html</t>
+  </si>
+  <si>
+    <t>IMS lists no pebble mills, so this is a sourcing page: a sourcing block replaces the IMS listing (new builder option), the hero and closing search point at IMS's full mill category, and business copy that assumes stock is rewritten. It links IPP's new ball mill page by relative path (resolves once P29 is published) and names the TEMA vibratory mill whose listing accepts pebble media. Rebuild the page if IMS lists a pebble mill.</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Pellet</t>
+  </si>
+  <si>
+    <t>Pellet Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/pellet/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pellet</t>
+  </si>
+  <si>
+    <t>pelletizer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/pellet/</t>
+  </si>
+  <si>
+    <t>equipment/mill/pellet/INTERNAL-REVIEW-pellet.html</t>
+  </si>
+  <si>
+    <t>IMS's pellet mill category holds a Black Clawson underwater pelletizing system (Gala spin dryer, MAAG gear pump, Kenics exchanger) and a Baker Perkins centrifugal pelletizer, not ring-die or flat-die pellet mills, so the page is built as 'Pelletizers'. Feed, wood and biomass pellet mill demand gets one FAQ (sourcing) and is otherwise excluded. A hero card opens IMS's site-wide pelletizer search (waterslide and Rieter (Maag) strand units in the plastics categories).</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>Roll</t>
+  </si>
+  <si>
+    <t>Roll Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/roll/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/roll</t>
+  </si>
+  <si>
+    <t>roll mill</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/roll/</t>
+  </si>
+  <si>
+    <t>equipment/mill/roll/INTERNAL-REVIEW-roll.html</t>
+  </si>
+  <si>
+    <t>Two-roll mills (lab, Farrel, chrome, unused and carbon steel) and a Gundlach 4080S two-roll crusher, with good used and unused condition tabs. Grain roller mills, three-roll mills and metal rolling mills are excluded. IMS spells the maker 'Farrell'; the copy uses Farrel. The crusher's previous use stays off the page.</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>Shot And Sand</t>
+  </si>
+  <si>
+    <t>Shot and Sand Mills</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mill/shot-and-sand/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/shot-and-sand</t>
+  </si>
+  <si>
+    <t>bead mill</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mill/shot-and-sand/</t>
+  </si>
+  <si>
+    <t>equipment/mill/shot-and-sand/INTERNAL-REVIEW-shot-and-sand.html</t>
+  </si>
+  <si>
+    <t>Built as 'Bead &amp; Sand Mills' from IMS's shot and sand category: Netzsch LMC, LME and LMJ, WAB Dyno-Mill, Asada, FrymaKoruma and Drais bead mills, Moorhouse and Premier-type sandmill systems and Union Process Szegvari attritors, plus rebuilt Netzsch seals and an unused drive part. Type tabs and Netzsch, WAB and Asada manufacturer tabs; no condition tabs, since the refurbished and unused items are parts. Bead mill homogenizers and basket mills are excluded; media-volume fields, hazardous-area wording and throughput figures stay off the page.</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>Mixer-Banbury</t>
+  </si>
+  <si>
+    <t>Banbury Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/banbury-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/banbury-mixer</t>
+  </si>
+  <si>
     <t>Not started</t>
   </si>
   <si>
-    <t>equipment/mill/kady/INTERNAL-REVIEW-kady.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 1 unit on IMS.</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>Pebble</t>
-  </si>
-  <si>
-    <t>Pebble Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/pebble/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pebble</t>
-  </si>
-  <si>
-    <t>equipment/mill/pebble/INTERNAL-REVIEW-pebble.html</t>
-  </si>
-  <si>
-    <t>IMS shows 0 units. The page will be a sourcing page with no listing.</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>Pellet</t>
-  </si>
-  <si>
-    <t>Pellet Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/pellet/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/pellet</t>
-  </si>
-  <si>
-    <t>equipment/mill/pellet/INTERNAL-REVIEW-pellet.html</t>
+    <t>equipment/mixer/banbury-mixer/INTERNAL-REVIEW-banbury-mixer.html</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>Mixer-Charge Can and Pony</t>
+  </si>
+  <si>
+    <t>Charge Can and Pony Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/charge-can-and-pony-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/charge-can-and-pony-mixer</t>
+  </si>
+  <si>
+    <t>equipment/mixer/charge-can-and-pony-mixer/INTERNAL-REVIEW-charge-can-and-pony-mixer.html</t>
+  </si>
+  <si>
+    <t>Thin inventory: 4 units.</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Mixer-Disperser</t>
+  </si>
+  <si>
+    <t>Disperser Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/disperser-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/disperser-mixer</t>
+  </si>
+  <si>
+    <t>equipment/mixer/disperser-mixer/INTERNAL-REVIEW-disperser-mixer.html</t>
+  </si>
+  <si>
+    <t>The IMS disperser search also returns a batch-type agitated reactor; it is excluded from the page.</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>Mixer-Munson and Rotating</t>
+  </si>
+  <si>
+    <t>Munson and Rotary Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/munson-rotary-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/munson-rotary-mixer</t>
+  </si>
+  <si>
+    <t>equipment/mixer/munson-rotary-mixer/INTERNAL-REVIEW-munson-rotary-mixer.html</t>
   </si>
   <si>
     <t>Thin inventory: 2 units.</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>Roll</t>
-  </si>
-  <si>
-    <t>Roll Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/roll/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/roll</t>
-  </si>
-  <si>
-    <t>equipment/mill/roll/INTERNAL-REVIEW-roll.html</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>Shot And Sand</t>
-  </si>
-  <si>
-    <t>Shot and Sand Mills</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mill/shot-and-sand/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/mill/shot-and-sand</t>
-  </si>
-  <si>
-    <t>equipment/mill/shot-and-sand/INTERNAL-REVIEW-shot-and-sand.html</t>
-  </si>
-  <si>
-    <t>IMS Mill &gt; Shot And Sand (33 listings). IMS also has a separate Mixer-Shot and Sand type, so check the entity overlap.</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>Mixer-Banbury</t>
-  </si>
-  <si>
-    <t>Banbury Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/banbury-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/banbury-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/banbury-mixer/INTERNAL-REVIEW-banbury-mixer.html</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>Mixer-Charge Can and Pony</t>
-  </si>
-  <si>
-    <t>Charge Can and Pony Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/charge-can-and-pony-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/charge-can-and-pony-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/charge-can-and-pony-mixer/INTERNAL-REVIEW-charge-can-and-pony-mixer.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 4 units.</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>Mixer-Disperser</t>
-  </si>
-  <si>
-    <t>Disperser Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/disperser-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/disperser-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/disperser-mixer/INTERNAL-REVIEW-disperser-mixer.html</t>
-  </si>
-  <si>
-    <t>The IMS disperser search also returns a batch-type agitated reactor; it is excluded from the page.</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>Mixer-Munson and Rotating</t>
-  </si>
-  <si>
-    <t>Munson and Rotary Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/munson-rotary-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/munson-rotary-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/munson-rotary-mixer/INTERNAL-REVIEW-munson-rotary-mixer.html</t>
   </si>
   <si>
     <t>Summary</t>
@@ -4266,7 +4302,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="36" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>313</v>
       </c>
@@ -4291,50 +4327,62 @@
       <c r="H36" s="3">
         <v>1</v>
       </c>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="3"/>
+      <c r="I36" s="3">
+        <v>1</v>
+      </c>
+      <c r="J36" s="3">
+        <v>1</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="L36" s="3">
+        <v>50</v>
+      </c>
       <c r="M36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="R36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="T36" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U36" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V36" s="4"/>
+      <c r="V36" s="5" t="s">
+        <v>319</v>
+      </c>
       <c r="W36" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="X36" s="4"/>
+        <v>320</v>
+      </c>
+      <c r="X36" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y36" s="7" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="37" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B37" s="3">
         <v>7</v>
@@ -4343,64 +4391,76 @@
         <v>295</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
       </c>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="3"/>
+      <c r="I37" s="3">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="L37" s="3">
+        <v>80</v>
+      </c>
       <c r="M37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="R37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="T37" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U37" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V37" s="4"/>
+      <c r="V37" s="5" t="s">
+        <v>328</v>
+      </c>
       <c r="W37" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="X37" s="4"/>
+        <v>329</v>
+      </c>
+      <c r="X37" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y37" s="7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="38" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B38" s="3">
         <v>7</v>
@@ -4409,64 +4469,76 @@
         <v>295</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="H38" s="3">
         <v>2</v>
       </c>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="3"/>
+      <c r="I38" s="3">
+        <v>2</v>
+      </c>
+      <c r="J38" s="3">
+        <v>2</v>
+      </c>
+      <c r="K38" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="L38" s="3">
+        <v>600</v>
+      </c>
       <c r="M38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="N38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="R38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="T38" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U38" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V38" s="4"/>
+      <c r="V38" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="W38" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="X38" s="4"/>
+        <v>338</v>
+      </c>
+      <c r="X38" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y38" s="7" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="39" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B39" s="3">
         <v>7</v>
@@ -4475,62 +4547,76 @@
         <v>295</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="H39" s="3">
         <v>6</v>
       </c>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="3"/>
+      <c r="I39" s="3">
+        <v>6</v>
+      </c>
+      <c r="J39" s="3">
+        <v>5</v>
+      </c>
+      <c r="K39" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="L39" s="3">
+        <v>150</v>
+      </c>
       <c r="M39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="R39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="T39" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U39" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V39" s="4"/>
+      <c r="V39" s="5" t="s">
+        <v>346</v>
+      </c>
       <c r="W39" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="X39" s="4"/>
-      <c r="Y39" s="7"/>
-    </row>
-    <row r="40" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>347</v>
+      </c>
+      <c r="X39" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B40" s="3">
         <v>7</v>
@@ -4539,80 +4625,92 @@
         <v>295</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="H40" s="3">
         <v>33</v>
       </c>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
-      <c r="K40" s="4"/>
-      <c r="L40" s="3"/>
+      <c r="I40" s="3">
+        <v>33</v>
+      </c>
+      <c r="J40" s="3">
+        <v>33</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="L40" s="3">
+        <v>250</v>
+      </c>
       <c r="M40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="N40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="R40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="S40" s="3" t="s">
-        <v>318</v>
+        <v>33</v>
       </c>
       <c r="T40" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U40" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V40" s="4"/>
+      <c r="V40" s="5" t="s">
+        <v>355</v>
+      </c>
       <c r="W40" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="X40" s="4"/>
+        <v>356</v>
+      </c>
+      <c r="X40" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y40" s="7" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
     </row>
     <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="B41" s="3">
         <v>8</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="H41" s="3">
         <v>9</v>
@@ -4622,25 +4720,25 @@
       <c r="K41" s="4"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4651,30 +4749,30 @@
       </c>
       <c r="V41" s="4"/>
       <c r="W41" s="4" t="s">
-        <v>353</v>
+        <v>364</v>
       </c>
       <c r="X41" s="4"/>
       <c r="Y41" s="7"/>
     </row>
     <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>355</v>
+        <v>366</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>356</v>
+        <v>367</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>357</v>
+        <v>368</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
@@ -4684,25 +4782,25 @@
       <c r="K42" s="4"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4713,32 +4811,32 @@
       </c>
       <c r="V42" s="4"/>
       <c r="W42" s="4" t="s">
-        <v>359</v>
+        <v>370</v>
       </c>
       <c r="X42" s="4"/>
       <c r="Y42" s="7" t="s">
-        <v>360</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>361</v>
+        <v>372</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>362</v>
+        <v>373</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>365</v>
+        <v>376</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
@@ -4748,25 +4846,25 @@
       <c r="K43" s="4"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4777,32 +4875,32 @@
       </c>
       <c r="V43" s="4"/>
       <c r="W43" s="4" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="X43" s="4"/>
       <c r="Y43" s="7" t="s">
-        <v>367</v>
+        <v>378</v>
       </c>
     </row>
     <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>370</v>
+        <v>381</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>372</v>
+        <v>383</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
@@ -4812,25 +4910,25 @@
       <c r="K44" s="4"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4841,11 +4939,11 @@
       </c>
       <c r="V44" s="4"/>
       <c r="W44" s="4" t="s">
-        <v>373</v>
+        <v>384</v>
       </c>
       <c r="X44" s="4"/>
       <c r="Y44" s="7" t="s">
-        <v>334</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -4988,22 +5086,27 @@
     <hyperlink ref="V35" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
     <hyperlink ref="F36" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
     <hyperlink ref="G36" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="F37" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="G37" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="F38" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="G38" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="F39" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="G39" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
-    <hyperlink ref="F40" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
-    <hyperlink ref="G40" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
-    <hyperlink ref="F41" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
-    <hyperlink ref="G41" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
-    <hyperlink ref="F42" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
-    <hyperlink ref="G42" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
-    <hyperlink ref="F43" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
-    <hyperlink ref="G43" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
-    <hyperlink ref="F44" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
-    <hyperlink ref="G44" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="V36" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="F37" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="G37" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="V37" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="F38" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="G38" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="V38" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="F39" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="G39" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="V39" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="F40" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="G40" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="V40" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="F41" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="G41" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="F42" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="G42" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="F43" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="G43" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="F44" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="G44" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5023,25 +5126,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -5050,16 +5153,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -5068,16 +5171,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -5086,7 +5189,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -5095,7 +5198,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -5104,27 +5207,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>682</v>
+        <v>724</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -5133,11 +5236,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -5146,11 +5249,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5159,11 +5262,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -5172,11 +5275,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -5185,11 +5288,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -5198,11 +5301,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -5211,16 +5314,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.77500000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5228,16 +5331,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -5397,7 +5500,7 @@
       </c>
       <c r="C33" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A33,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D33" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A33,Pages!$U$5:$U$44,"Approved")</f>
@@ -5405,7 +5508,7 @@
       </c>
       <c r="E33" s="6" t="str">
         <f>IF(D33=B33,"Approved",IF(C33=B33,"Ready for client review",IF(C33&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A33,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -5445,15 +5548,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5461,7 +5564,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -5469,7 +5572,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -5477,7 +5580,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5485,7 +5588,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -5493,7 +5596,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5501,7 +5604,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -5509,7 +5612,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5517,28 +5620,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Tracker: batch 8 (P36-39) ready for client review; all 40 pages done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ipp-40-pages-status-tracker.xlsx
+++ b/docs/ipp-40-pages-status-tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dilbd\repos\ipp-updated\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4D0BB7-A446-4F86-AA3A-64ADA71C3B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F824E3B-F440-4965-A1E3-7AA3CC4CE40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="429">
   <si>
     <t>IPP Next 39 Priorities: Landing Page Status Tracker (40 pages)</t>
   </si>
@@ -1129,94 +1129,121 @@
     <t>https://ims.internationalprocessplants.com/inventory/search/equipment/banbury-mixer</t>
   </si>
   <si>
+    <t>banbury mixer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mixer/banbury-mixer/</t>
+  </si>
+  <si>
+    <t>equipment/mixer/banbury-mixer/INTERNAL-REVIEW-banbury-mixer.html</t>
+  </si>
+  <si>
+    <t>IMS's Banbury category holds no Banbury internal mixer: it lists a Mazzoni MSB-1600 amalgamator, Mazzoni TDS-150-N turbodispersers and Fabricated Products AC05M additive mixers, none with photos. The page is built as 'Banbury Mixers &amp; Amalgamators' and offers Banbury mixers through sourcing. 'amalgamator' searches are dental, and the turbodisperser is named but not defined because no reliable source describes it. An FAQ tells buyers that photos come with IPP's data sheet.</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>Mixer-Charge Can and Pony</t>
+  </si>
+  <si>
+    <t>Charge Can and Pony Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/charge-can-and-pony-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/charge-can-and-pony-mixer</t>
+  </si>
+  <si>
+    <t>planetary mixer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mixer/charge-can-and-pony-mixer/</t>
+  </si>
+  <si>
+    <t>equipment/mixer/charge-can-and-pony-mixer/INTERNAL-REVIEW-charge-can-and-pony-mixer.html</t>
+  </si>
+  <si>
+    <t>Built as 'Planetary &amp; Change Can Mixers' (IMS calls the category 'charge can and pony'): a titanium Ross HDM 150, a Ross PD-2 PowerMix planetary disperser, a Haagen-Rinau Unimax tri-homo mixer and a Drais FH80 change can vacuum mixer. The head term is foodservice-heavy, so stand-mixer brands and bakery terms are excluded. IMS's Haagen-Rinau can-size fields are wrong; the listing text's 600 by 430 mm is published.</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Mixer-Disperser</t>
+  </si>
+  <si>
+    <t>Disperser Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/disperser-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/disperser-mixer</t>
+  </si>
+  <si>
+    <t>disperser mixer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mixer/disperser-mixer/</t>
+  </si>
+  <si>
+    <t>equipment/mixer/disperser-mixer/INTERNAL-REVIEW-disperser-mixer.html</t>
+  </si>
+  <si>
+    <t>Ten dispersers in three type tabs: Morehouse-COWLES, Drais, Bowers and Fluid high-speed units; Abbe Dispersall, Fryma VME-500, Buhler twin-shaft and Joshua Greaves vacuum or multi-shaft systems; Barker &amp; Aspey tank-mount agitators. IMS's two non-disperser hits are left out. Comparison: high-speed dispersers vs rotor-stator high-shear mixers.</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>Mixer-Munson and Rotating</t>
+  </si>
+  <si>
+    <t>Munson and Rotary Mixers</t>
+  </si>
+  <si>
+    <t>https://internationalprocessplants.com/process-equipment/mixer/munson-rotary-mixer/</t>
+  </si>
+  <si>
+    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/munson-rotary-mixer</t>
+  </si>
+  <si>
+    <t>munson mixer</t>
+  </si>
+  <si>
+    <t>https://international-process-plants-update-one.vercel.app/equipment/mixer/munson-rotary-mixer/</t>
+  </si>
+  <si>
+    <t>equipment/mixer/munson-rotary-mixer/INTERNAL-REVIEW-munson-rotary-mixer.html</t>
+  </si>
+  <si>
+    <t>A Munson VIM368SS variable intensity (continuous) mixer and a rotating bowl blender. The Munson listing's missing-drive-gear note, its throughput figure and the bowl blender's impossible capacity field stay off the page; the data sheet covers condition. Comparison: Munson variable intensity vs rotary batch mixers (sourced to specification). 'rotary mixer' searches are mostly DJ mixers and are excluded.</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>Every figure on this sheet is a formula over the Pages sheet.</t>
+  </si>
+  <si>
+    <t>Measure</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Pages in scope</t>
+  </si>
+  <si>
+    <t>Ready for client review</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
     <t>Not started</t>
-  </si>
-  <si>
-    <t>equipment/mixer/banbury-mixer/INTERNAL-REVIEW-banbury-mixer.html</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>Mixer-Charge Can and Pony</t>
-  </si>
-  <si>
-    <t>Charge Can and Pony Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/charge-can-and-pony-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/charge-can-and-pony-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/charge-can-and-pony-mixer/INTERNAL-REVIEW-charge-can-and-pony-mixer.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 4 units.</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>Mixer-Disperser</t>
-  </si>
-  <si>
-    <t>Disperser Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/disperser-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/disperser-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/disperser-mixer/INTERNAL-REVIEW-disperser-mixer.html</t>
-  </si>
-  <si>
-    <t>The IMS disperser search also returns a batch-type agitated reactor; it is excluded from the page.</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>Mixer-Munson and Rotating</t>
-  </si>
-  <si>
-    <t>Munson and Rotary Mixers</t>
-  </si>
-  <si>
-    <t>https://internationalprocessplants.com/process-equipment/mixer/munson-rotary-mixer/</t>
-  </si>
-  <si>
-    <t>https://ims.internationalprocessplants.com/inventory/search/equipment/munson-rotary-mixer</t>
-  </si>
-  <si>
-    <t>equipment/mixer/munson-rotary-mixer/INTERNAL-REVIEW-munson-rotary-mixer.html</t>
-  </si>
-  <si>
-    <t>Thin inventory: 2 units.</t>
-  </si>
-  <si>
-    <t>Summary</t>
-  </si>
-  <si>
-    <t>Every figure on this sheet is a formula over the Pages sheet.</t>
-  </si>
-  <si>
-    <t>Measure</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Pages in scope</t>
-  </si>
-  <si>
-    <t>Ready for client review</t>
-  </si>
-  <si>
-    <t>In progress</t>
   </si>
   <si>
     <t>Blocked</t>
@@ -4692,7 +4719,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="41" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" ht="102" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>358</v>
       </c>
@@ -4715,235 +4742,285 @@
       <c r="H41" s="3">
         <v>9</v>
       </c>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="3"/>
+      <c r="I41" s="3">
+        <v>9</v>
+      </c>
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="L41" s="3">
+        <v>250</v>
+      </c>
       <c r="M41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="R41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="S41" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="T41" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U41" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V41" s="4"/>
+      <c r="V41" s="5" t="s">
+        <v>364</v>
+      </c>
       <c r="W41" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="X41" s="4"/>
-      <c r="Y41" s="7"/>
-    </row>
-    <row r="42" spans="1:25" ht="38.25" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+      <c r="X41" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y41" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B42" s="3">
         <v>8</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="H42" s="3">
         <v>4</v>
       </c>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="3"/>
+      <c r="I42" s="3">
+        <v>4</v>
+      </c>
+      <c r="J42" s="3">
+        <v>4</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="L42" s="3">
+        <v>1100</v>
+      </c>
       <c r="M42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="N42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="R42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="S42" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="T42" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U42" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V42" s="4"/>
+      <c r="V42" s="5" t="s">
+        <v>373</v>
+      </c>
       <c r="W42" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="X42" s="4"/>
+        <v>374</v>
+      </c>
+      <c r="X42" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y42" s="7" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="43" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B43" s="3">
         <v>8</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="H43" s="3">
         <v>12</v>
       </c>
-      <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="3"/>
+      <c r="I43" s="3">
+        <v>10</v>
+      </c>
+      <c r="J43" s="3">
+        <v>8</v>
+      </c>
+      <c r="K43" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="L43" s="3">
+        <v>150</v>
+      </c>
       <c r="M43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="O43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="R43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="T43" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U43" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V43" s="4"/>
+      <c r="V43" s="5" t="s">
+        <v>382</v>
+      </c>
       <c r="W43" s="4" t="s">
-        <v>377</v>
-      </c>
-      <c r="X43" s="4"/>
+        <v>383</v>
+      </c>
+      <c r="X43" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y43" s="7" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="44" spans="1:25" ht="25.5" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B44" s="3">
         <v>8</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="H44" s="3">
         <v>2</v>
       </c>
-      <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="3"/>
+      <c r="I44" s="3">
+        <v>2</v>
+      </c>
+      <c r="J44" s="3">
+        <v>2</v>
+      </c>
+      <c r="K44" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="L44" s="3">
+        <v>30</v>
+      </c>
       <c r="M44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="Q44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="R44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="S44" s="3" t="s">
-        <v>363</v>
+        <v>33</v>
       </c>
       <c r="T44" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
       <c r="U44" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="V44" s="4"/>
+      <c r="V44" s="5" t="s">
+        <v>391</v>
+      </c>
       <c r="W44" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="X44" s="4"/>
+        <v>392</v>
+      </c>
+      <c r="X44" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="Y44" s="7" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -5101,12 +5178,16 @@
     <hyperlink ref="V40" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
     <hyperlink ref="F41" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
     <hyperlink ref="G41" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
-    <hyperlink ref="F42" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
-    <hyperlink ref="G42" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
-    <hyperlink ref="F43" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
-    <hyperlink ref="G43" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
-    <hyperlink ref="F44" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
-    <hyperlink ref="G44" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="V41" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="F42" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="G42" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="V42" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="F43" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="G43" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="V43" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="F44" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="G44" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="V44" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5126,25 +5207,25 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTA(Pages!$A$5:$A$44)</f>
@@ -5153,16 +5234,16 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="B6" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B7" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"In progress")</f>
@@ -5171,16 +5252,16 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>363</v>
+        <v>401</v>
       </c>
       <c r="B8" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Not started")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="B9" s="6">
         <f>COUNTIF(Pages!$T$5:$T$44,"Blocked")</f>
@@ -5189,7 +5270,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>394</v>
+        <v>403</v>
       </c>
       <c r="B10" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Approved")</f>
@@ -5198,7 +5279,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>395</v>
+        <v>404</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTIF(Pages!$U$5:$U$44,"Changes requested")</f>
@@ -5207,27 +5288,27 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>396</v>
+        <v>405</v>
       </c>
       <c r="B12" s="6">
         <f>SUM(Pages!$I$5:$I$44)</f>
-        <v>724</v>
+        <v>749</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -5236,11 +5317,11 @@
       </c>
       <c r="B16" s="10">
         <f>COUNTIF(Pages!$M$5:$M$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C16" s="12">
         <f t="shared" ref="C16:C22" si="0">IF($B$5=0,0,B16/$B$5)</f>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -5249,11 +5330,11 @@
       </c>
       <c r="B17" s="10">
         <f>COUNTIF(Pages!$N$5:$N$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C17" s="12">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -5262,11 +5343,11 @@
       </c>
       <c r="B18" s="10">
         <f>COUNTIF(Pages!$O$5:$O$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C18" s="12">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -5275,11 +5356,11 @@
       </c>
       <c r="B19" s="10">
         <f>COUNTIF(Pages!$P$5:$P$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C19" s="12">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -5288,11 +5369,11 @@
       </c>
       <c r="B20" s="10">
         <f>COUNTIF(Pages!$Q$5:$Q$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C20" s="12">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -5301,11 +5382,11 @@
       </c>
       <c r="B21" s="10">
         <f>COUNTIF(Pages!$R$5:$R$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C21" s="12">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -5314,16 +5395,16 @@
       </c>
       <c r="B22" s="10">
         <f>COUNTIF(Pages!$S$5:$S$44,"Done")</f>
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C22" s="12">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -5331,16 +5412,16 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>401</v>
+        <v>410</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>402</v>
+        <v>411</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>403</v>
+        <v>412</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -5521,7 +5602,7 @@
       </c>
       <c r="C34" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A34,Pages!$T$5:$T$44,"Ready for client review")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D34" s="10">
         <f>COUNTIFS(Pages!$B$5:$B$44,A34,Pages!$U$5:$U$44,"Approved")</f>
@@ -5529,7 +5610,7 @@
       </c>
       <c r="E34" s="6" t="str">
         <f>IF(D34=B34,"Approved",IF(C34=B34,"Ready for client review",IF(C34&gt;0,"In progress",IF(COUNTIFS(Pages!$B$5:$B$44,A34,Pages!$T$5:$T$44,"In progress")&gt;0,"In progress","Not started"))))</f>
-        <v>Not started</v>
+        <v>Ready for client review</v>
       </c>
     </row>
   </sheetData>
@@ -5548,15 +5629,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>406</v>
+        <v>415</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5564,7 +5645,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>407</v>
+        <v>416</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -5572,7 +5653,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>408</v>
+        <v>417</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -5580,7 +5661,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>409</v>
+        <v>418</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5588,7 +5669,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>410</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -5596,7 +5677,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5604,7 +5685,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>412</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -5612,7 +5693,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>413</v>
+        <v>422</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
@@ -5620,28 +5701,28 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>414</v>
+        <v>423</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>415</v>
+        <v>424</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>416</v>
+        <v>425</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>417</v>
+        <v>426</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>418</v>
+        <v>427</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>419</v>
+        <v>428</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>37</v>

</xml_diff>